<commit_message>
extract index case numbers and updating analysis to estimate contacts per index case across exposures
</commit_message>
<xml_diff>
--- a/data/sar_extraction.xlsx
+++ b/data/sar_extraction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ginacuomo-dannenburg/Documents/code/bvd-contacts/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5835AF9F-3672-8C46-AF70-EF63C7671322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D90E44-B6D5-C94F-B275-E5BE547FEC2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <sheet name="exposure_mapping_wip" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">data_me!$S$1:$S$1009</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">data_me!$T$1:$T$1009</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="209">
   <si>
     <t>first_author</t>
   </si>
@@ -812,6 +812,9 @@
   <si>
     <t>Combined into one indirect exposure</t>
   </si>
+  <si>
+    <t>num_index</t>
+  </si>
 </sst>
 </file>
 
@@ -7847,7 +7850,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1009"/>
+  <dimension ref="A1:AB1009"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="15.6640625" customWidth="1"/>
@@ -7855,14 +7858,14 @@
     <col min="9" max="9" width="51" customWidth="1"/>
     <col min="12" max="12" width="21.1640625" customWidth="1"/>
     <col min="15" max="15" width="14.5" customWidth="1"/>
-    <col min="16" max="16" width="15.5" customWidth="1"/>
-    <col min="17" max="17" width="15.6640625" customWidth="1"/>
-    <col min="18" max="18" width="51" customWidth="1"/>
-    <col min="21" max="21" width="112.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="16384" width="12.6640625" style="42"/>
+    <col min="16" max="17" width="15.5" customWidth="1"/>
+    <col min="18" max="18" width="15.6640625" customWidth="1"/>
+    <col min="19" max="19" width="51" customWidth="1"/>
+    <col min="22" max="22" width="112.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="12.6640625" style="42"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27">
+    <row r="1" spans="1:28" ht="16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7912,28 +7915,31 @@
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="V1" s="41"/>
       <c r="W1" s="41"/>
       <c r="X1" s="41"/>
       <c r="Y1" s="41"/>
       <c r="Z1" s="41"/>
       <c r="AA1" s="41"/>
-    </row>
-    <row r="2" spans="1:27" ht="15.75" customHeight="1">
+      <c r="AB1" s="41"/>
+    </row>
+    <row r="2" spans="1:28" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>17</v>
       </c>
@@ -7982,20 +7988,23 @@
       <c r="P2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Q2" s="7">
+      <c r="Q2" s="4">
+        <v>34</v>
+      </c>
+      <c r="R2" s="7">
         <v>9</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="S2" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T2" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:27" ht="15.75" customHeight="1">
+      <c r="U2" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>17</v>
       </c>
@@ -8044,20 +8053,23 @@
       <c r="P3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Q3" s="7">
+      <c r="Q3" s="4">
+        <v>34</v>
+      </c>
+      <c r="R3" s="7">
         <v>9</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="S3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="S3" s="4" t="b">
+      <c r="T3" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T3" s="4" t="b">
+      <c r="U3" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="15.75" customHeight="1">
+    <row r="4" spans="1:28" ht="15.75" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -8106,20 +8118,23 @@
       <c r="P4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Q4" s="7">
+      <c r="Q4" s="4">
+        <v>34</v>
+      </c>
+      <c r="R4" s="7">
         <v>9</v>
       </c>
-      <c r="R4" s="4" t="s">
+      <c r="S4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="S4" s="4" t="b">
+      <c r="T4" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T4" s="4" t="b">
+      <c r="U4" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="15.75" customHeight="1">
+    <row r="5" spans="1:28" ht="15.75" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>17</v>
       </c>
@@ -8168,20 +8183,23 @@
       <c r="P5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Q5" s="7">
+      <c r="Q5" s="4">
+        <v>34</v>
+      </c>
+      <c r="R5" s="7">
         <v>9</v>
       </c>
-      <c r="R5" s="4" t="s">
+      <c r="S5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S5" s="4" t="b">
+      <c r="T5" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T5" s="4" t="b">
+      <c r="U5" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="15.75" customHeight="1">
+    <row r="6" spans="1:28" ht="15.75" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>17</v>
       </c>
@@ -8230,20 +8248,23 @@
       <c r="P6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Q6" s="7">
+      <c r="Q6" s="4">
+        <v>34</v>
+      </c>
+      <c r="R6" s="7">
         <v>9</v>
       </c>
-      <c r="R6" s="4" t="s">
+      <c r="S6" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="S6" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T6" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:27" ht="15.75" customHeight="1">
+      <c r="U6" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="15.75" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>30</v>
       </c>
@@ -8292,20 +8313,24 @@
       <c r="P7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="Q7" s="7">
+      <c r="Q7" s="4">
+        <f>117+27</f>
+        <v>144</v>
+      </c>
+      <c r="R7" s="7">
         <v>9</v>
       </c>
-      <c r="R7" s="4" t="s">
+      <c r="S7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="S7" s="4" t="b">
+      <c r="T7" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T7" s="4" t="b">
+      <c r="U7" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="15.75" customHeight="1">
+    <row r="8" spans="1:28" ht="15.75" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>30</v>
       </c>
@@ -8354,20 +8379,23 @@
       <c r="P8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="Q8" s="7">
+      <c r="Q8" s="4">
+        <v>144</v>
+      </c>
+      <c r="R8" s="7">
         <v>9</v>
       </c>
-      <c r="R8" s="4" t="s">
+      <c r="S8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="S8" s="4" t="b">
+      <c r="T8" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T8" s="4" t="b">
+      <c r="U8" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="15.75" customHeight="1">
+    <row r="9" spans="1:28" ht="15.75" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>30</v>
       </c>
@@ -8416,20 +8444,23 @@
       <c r="P9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="7">
+      <c r="Q9" s="4">
+        <v>144</v>
+      </c>
+      <c r="R9" s="7">
         <v>9</v>
       </c>
-      <c r="R9" s="4" t="s">
+      <c r="S9" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="S9" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T9" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:27" ht="15.75" customHeight="1">
+      <c r="U9" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" ht="15.75" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>43</v>
       </c>
@@ -8478,20 +8509,23 @@
       <c r="P10" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="Q10" s="7">
+      <c r="Q10" s="4">
+        <v>30</v>
+      </c>
+      <c r="R10" s="7">
         <v>9</v>
       </c>
-      <c r="R10" s="4" t="s">
+      <c r="S10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="S10" s="4" t="b">
+      <c r="T10" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T10" s="4" t="b">
+      <c r="U10" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:27" ht="15.75" customHeight="1">
+    <row r="11" spans="1:28" ht="15.75" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>43</v>
       </c>
@@ -8540,20 +8574,23 @@
       <c r="P11" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="Q11" s="7">
+      <c r="Q11" s="4">
+        <v>30</v>
+      </c>
+      <c r="R11" s="7">
         <v>9</v>
       </c>
-      <c r="R11" s="4" t="s">
+      <c r="S11" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="S11" s="4" t="b">
+      <c r="T11" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T11" s="4" t="b">
+      <c r="U11" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:27" ht="15.75" customHeight="1">
+    <row r="12" spans="1:28" ht="15.75" customHeight="1">
       <c r="A12" s="4" t="s">
         <v>43</v>
       </c>
@@ -8602,20 +8639,23 @@
       <c r="P12" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="Q12" s="7">
+      <c r="Q12" s="4">
+        <v>30</v>
+      </c>
+      <c r="R12" s="7">
         <v>9</v>
       </c>
-      <c r="R12" s="4" t="s">
+      <c r="S12" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="S12" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T12" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:27" ht="15.75" customHeight="1">
+      <c r="U12" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" ht="15.75" customHeight="1">
       <c r="A13" s="4" t="s">
         <v>54</v>
       </c>
@@ -8664,20 +8704,23 @@
       <c r="P13" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q13" s="7">
+      <c r="Q13" s="4">
+        <v>150</v>
+      </c>
+      <c r="R13" s="7">
         <v>9</v>
       </c>
-      <c r="R13" s="4" t="s">
+      <c r="S13" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="S13" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T13" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:27" ht="15.75" customHeight="1">
+      <c r="U13" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" ht="15.75" customHeight="1">
       <c r="A14" s="4" t="s">
         <v>54</v>
       </c>
@@ -8726,20 +8769,23 @@
       <c r="P14" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q14" s="7">
+      <c r="Q14" s="4">
+        <v>150</v>
+      </c>
+      <c r="R14" s="7">
         <v>9</v>
       </c>
-      <c r="R14" s="4" t="s">
+      <c r="S14" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="S14" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T14" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:27" ht="15.75" customHeight="1">
+      <c r="U14" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" ht="15.75" customHeight="1">
       <c r="A15" s="4" t="s">
         <v>54</v>
       </c>
@@ -8788,20 +8834,23 @@
       <c r="P15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q15" s="7">
+      <c r="Q15" s="4">
+        <v>150</v>
+      </c>
+      <c r="R15" s="7">
         <v>9</v>
       </c>
-      <c r="R15" s="4" t="s">
+      <c r="S15" s="4" t="s">
         <v>64</v>
-      </c>
-      <c r="S15" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T15" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:27" ht="15.75" customHeight="1">
+      <c r="U15" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" ht="15.75" customHeight="1">
       <c r="A16" s="4" t="s">
         <v>54</v>
       </c>
@@ -8850,20 +8899,23 @@
       <c r="P16" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q16" s="7">
+      <c r="Q16" s="4">
+        <v>150</v>
+      </c>
+      <c r="R16" s="7">
         <v>9</v>
       </c>
-      <c r="R16" s="4" t="s">
+      <c r="S16" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="S16" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T16" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U16" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" ht="15.75" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>54</v>
       </c>
@@ -8912,20 +8964,23 @@
       <c r="P17" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q17" s="7">
+      <c r="Q17" s="4">
+        <v>150</v>
+      </c>
+      <c r="R17" s="7">
         <v>9</v>
       </c>
-      <c r="R17" s="4" t="s">
+      <c r="S17" s="4" t="s">
         <v>66</v>
-      </c>
-      <c r="S17" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T17" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U17" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" ht="15.75" customHeight="1">
       <c r="A18" s="4" t="s">
         <v>54</v>
       </c>
@@ -8974,20 +9029,23 @@
       <c r="P18" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q18" s="7">
+      <c r="Q18" s="4">
+        <v>150</v>
+      </c>
+      <c r="R18" s="7">
         <v>9</v>
       </c>
-      <c r="R18" s="4" t="s">
+      <c r="S18" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="S18" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T18" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U18" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" ht="15.75" customHeight="1">
       <c r="A19" s="4" t="s">
         <v>54</v>
       </c>
@@ -9036,20 +9094,23 @@
       <c r="P19" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q19" s="7">
+      <c r="Q19" s="4">
+        <v>150</v>
+      </c>
+      <c r="R19" s="7">
         <v>9</v>
       </c>
-      <c r="R19" s="4" t="s">
+      <c r="S19" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="S19" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T19" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U19" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="s">
         <v>54</v>
       </c>
@@ -9098,20 +9159,23 @@
       <c r="P20" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="Q20" s="7">
+      <c r="Q20" s="4">
+        <v>150</v>
+      </c>
+      <c r="R20" s="7">
         <v>9</v>
       </c>
-      <c r="R20" s="4" t="s">
+      <c r="S20" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="S20" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T20" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U20" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" ht="15.75" customHeight="1">
       <c r="A21" s="9" t="s">
         <v>54</v>
       </c>
@@ -9160,23 +9224,26 @@
       <c r="P21" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="Q21" s="9">
+      <c r="Q21" s="4">
+        <v>150</v>
+      </c>
+      <c r="R21" s="9">
         <v>9</v>
       </c>
-      <c r="R21" s="9" t="s">
+      <c r="S21" s="9" t="s">
         <v>64</v>
-      </c>
-      <c r="S21" s="9" t="b">
-        <v>1</v>
       </c>
       <c r="T21" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="U21" s="9" t="s">
+      <c r="U21" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V21" s="9" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="15.75" customHeight="1">
+    <row r="22" spans="1:22" ht="15.75" customHeight="1">
       <c r="A22" s="9" t="s">
         <v>54</v>
       </c>
@@ -9225,23 +9292,26 @@
       <c r="P22" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="Q22" s="9">
+      <c r="Q22" s="4">
+        <v>150</v>
+      </c>
+      <c r="R22" s="9">
         <v>9</v>
       </c>
-      <c r="R22" s="9" t="s">
+      <c r="S22" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="S22" s="9" t="b">
-        <v>1</v>
       </c>
       <c r="T22" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="U22" s="9" t="s">
+      <c r="U22" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V22" s="9" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="15.75" customHeight="1">
+    <row r="23" spans="1:22" ht="15.75" customHeight="1">
       <c r="A23" s="9" t="s">
         <v>54</v>
       </c>
@@ -9290,23 +9360,26 @@
       <c r="P23" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="Q23" s="9">
+      <c r="Q23" s="4">
+        <v>150</v>
+      </c>
+      <c r="R23" s="9">
         <v>9</v>
       </c>
-      <c r="R23" s="9" t="s">
+      <c r="S23" s="9" t="s">
         <v>146</v>
-      </c>
-      <c r="S23" s="9" t="b">
-        <v>1</v>
       </c>
       <c r="T23" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="U23" s="9" t="s">
+      <c r="U23" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V23" s="9" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="15.75" customHeight="1">
+    <row r="24" spans="1:22" ht="15.75" customHeight="1">
       <c r="A24" s="9" t="s">
         <v>54</v>
       </c>
@@ -9355,23 +9428,26 @@
       <c r="P24" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="Q24" s="9">
+      <c r="Q24" s="4">
+        <v>150</v>
+      </c>
+      <c r="R24" s="9">
         <v>9</v>
       </c>
-      <c r="R24" s="9" t="s">
+      <c r="S24" s="9" t="s">
         <v>147</v>
-      </c>
-      <c r="S24" s="9" t="b">
-        <v>1</v>
       </c>
       <c r="T24" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="U24" s="9" t="s">
+      <c r="U24" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V24" s="9" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:21" ht="15.75" customHeight="1">
+    <row r="25" spans="1:22" ht="15.75" customHeight="1">
       <c r="A25" s="35" t="s">
         <v>70</v>
       </c>
@@ -9421,22 +9497,25 @@
         <v>62</v>
       </c>
       <c r="Q25" s="35">
+        <v>27</v>
+      </c>
+      <c r="R25" s="35">
         <v>9</v>
       </c>
-      <c r="R25" s="35" t="s">
+      <c r="S25" s="35" t="s">
         <v>76</v>
-      </c>
-      <c r="S25" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T25" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U25" s="40" t="s">
+      <c r="U25" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V25" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="15.75" customHeight="1">
+    <row r="26" spans="1:22" ht="15.75" customHeight="1">
       <c r="A26" s="35" t="s">
         <v>70</v>
       </c>
@@ -9486,22 +9565,25 @@
         <v>62</v>
       </c>
       <c r="Q26" s="35">
+        <v>27</v>
+      </c>
+      <c r="R26" s="35">
         <v>9</v>
       </c>
-      <c r="R26" s="35" t="s">
+      <c r="S26" s="35" t="s">
         <v>77</v>
-      </c>
-      <c r="S26" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T26" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U26" s="40" t="s">
+      <c r="U26" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V26" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="27" spans="1:21" ht="15.75" customHeight="1">
+    <row r="27" spans="1:22" ht="15.75" customHeight="1">
       <c r="A27" s="35" t="s">
         <v>70</v>
       </c>
@@ -9551,22 +9633,25 @@
         <v>62</v>
       </c>
       <c r="Q27" s="35">
+        <v>27</v>
+      </c>
+      <c r="R27" s="35">
         <v>9</v>
       </c>
-      <c r="R27" s="35" t="s">
+      <c r="S27" s="35" t="s">
         <v>78</v>
-      </c>
-      <c r="S27" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T27" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U27" s="40" t="s">
+      <c r="U27" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V27" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="28" spans="1:21" ht="15.75" customHeight="1">
+    <row r="28" spans="1:22" ht="15.75" customHeight="1">
       <c r="A28" s="35" t="s">
         <v>70</v>
       </c>
@@ -9616,22 +9701,25 @@
         <v>62</v>
       </c>
       <c r="Q28" s="35">
+        <v>27</v>
+      </c>
+      <c r="R28" s="35">
         <v>9</v>
       </c>
-      <c r="R28" s="35" t="s">
+      <c r="S28" s="35" t="s">
         <v>79</v>
-      </c>
-      <c r="S28" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T28" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U28" s="40" t="s">
+      <c r="U28" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V28" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="29" spans="1:21" ht="15.75" customHeight="1">
+    <row r="29" spans="1:22" ht="15.75" customHeight="1">
       <c r="A29" s="35" t="s">
         <v>70</v>
       </c>
@@ -9681,22 +9769,25 @@
         <v>62</v>
       </c>
       <c r="Q29" s="35">
+        <v>27</v>
+      </c>
+      <c r="R29" s="35">
         <v>9</v>
       </c>
-      <c r="R29" s="35" t="s">
+      <c r="S29" s="35" t="s">
         <v>80</v>
-      </c>
-      <c r="S29" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T29" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U29" s="40" t="s">
+      <c r="U29" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V29" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="15.75" customHeight="1">
+    <row r="30" spans="1:22" ht="15.75" customHeight="1">
       <c r="A30" s="35" t="s">
         <v>70</v>
       </c>
@@ -9746,22 +9837,25 @@
         <v>62</v>
       </c>
       <c r="Q30" s="35">
+        <v>27</v>
+      </c>
+      <c r="R30" s="35">
         <v>9</v>
       </c>
-      <c r="R30" s="35" t="s">
+      <c r="S30" s="35" t="s">
         <v>81</v>
-      </c>
-      <c r="S30" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T30" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U30" s="40" t="s">
+      <c r="U30" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V30" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="15.75" customHeight="1">
+    <row r="31" spans="1:22" ht="15.75" customHeight="1">
       <c r="A31" s="35" t="s">
         <v>70</v>
       </c>
@@ -9811,22 +9905,25 @@
         <v>62</v>
       </c>
       <c r="Q31" s="35">
+        <v>27</v>
+      </c>
+      <c r="R31" s="35">
         <v>9</v>
       </c>
-      <c r="R31" s="35" t="s">
+      <c r="S31" s="35" t="s">
         <v>82</v>
-      </c>
-      <c r="S31" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T31" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U31" s="40" t="s">
+      <c r="U31" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V31" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="15.75" customHeight="1">
+    <row r="32" spans="1:22" ht="15.75" customHeight="1">
       <c r="A32" s="4" t="s">
         <v>83</v>
       </c>
@@ -9876,19 +9973,22 @@
         <v>88</v>
       </c>
       <c r="Q32" s="4">
+        <v>71</v>
+      </c>
+      <c r="R32" s="4">
         <v>9</v>
       </c>
-      <c r="R32" s="4" t="s">
+      <c r="S32" s="4" t="s">
         <v>87</v>
-      </c>
-      <c r="S32" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T32" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U32" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" ht="15.75" customHeight="1">
       <c r="A33" s="4" t="s">
         <v>83</v>
       </c>
@@ -9938,19 +10038,22 @@
         <v>88</v>
       </c>
       <c r="Q33" s="4">
+        <v>71</v>
+      </c>
+      <c r="R33" s="4">
         <v>9</v>
       </c>
-      <c r="R33" s="4" t="s">
+      <c r="S33" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="S33" s="4" t="b">
+      <c r="T33" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T33" s="4" t="b">
+      <c r="U33" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:21" ht="15.75" customHeight="1">
+    <row r="34" spans="1:22" ht="15.75" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>83</v>
       </c>
@@ -10000,19 +10103,22 @@
         <v>88</v>
       </c>
       <c r="Q34" s="4">
+        <v>71</v>
+      </c>
+      <c r="R34" s="4">
         <v>9</v>
       </c>
-      <c r="R34" s="4" t="s">
+      <c r="S34" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="S34" s="4" t="b">
+      <c r="T34" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T34" s="4" t="b">
+      <c r="U34" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:21" ht="15.75" customHeight="1">
+    <row r="35" spans="1:22" ht="15.75" customHeight="1">
       <c r="A35" s="4" t="s">
         <v>92</v>
       </c>
@@ -10061,20 +10167,23 @@
       <c r="P35" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="Q35" s="4" t="s">
+      <c r="Q35" s="4">
+        <v>27</v>
+      </c>
+      <c r="R35" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="R35" s="4" t="s">
+      <c r="S35" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="S35" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T35" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U35" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" ht="15.75" customHeight="1">
       <c r="A36" s="4" t="s">
         <v>92</v>
       </c>
@@ -10123,23 +10232,26 @@
       <c r="P36" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="Q36" s="4" t="s">
+      <c r="Q36" s="4">
+        <v>27</v>
+      </c>
+      <c r="R36" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="R36" s="4" t="s">
+      <c r="S36" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="S36" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T36" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="U36" s="4" t="s">
+      <c r="U36" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="V36" s="4" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="37" spans="1:21" ht="15.75" customHeight="1">
+    <row r="37" spans="1:22" ht="15.75" customHeight="1">
       <c r="A37" s="4" t="s">
         <v>92</v>
       </c>
@@ -10188,23 +10300,26 @@
       <c r="P37" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="Q37" s="4" t="s">
+      <c r="Q37" s="4">
+        <v>27</v>
+      </c>
+      <c r="R37" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="R37" s="4" t="s">
+      <c r="S37" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="S37" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T37" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="U37" s="4" t="s">
+      <c r="U37" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="V37" s="4" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="38" spans="1:21" ht="15.75" customHeight="1">
+    <row r="38" spans="1:22" ht="15.75" customHeight="1">
       <c r="A38" s="4" t="s">
         <v>101</v>
       </c>
@@ -10253,20 +10368,23 @@
       <c r="P38" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="Q38" s="4" t="s">
+      <c r="Q38" s="4">
+        <v>990</v>
+      </c>
+      <c r="R38" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="R38" s="4" t="s">
+      <c r="S38" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="S38" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T38" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U38" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" ht="15.75" customHeight="1">
       <c r="A39" s="4" t="s">
         <v>101</v>
       </c>
@@ -10315,23 +10433,26 @@
       <c r="P39" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="Q39" s="4" t="s">
+      <c r="Q39" s="4">
+        <v>990</v>
+      </c>
+      <c r="R39" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="R39" s="4" t="s">
+      <c r="S39" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="S39" s="4" t="b">
+      <c r="T39" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T39" s="4" t="b">
+      <c r="U39" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="U39" s="4" t="s">
+      <c r="V39" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="40" spans="1:21" ht="15.75" customHeight="1">
+    <row r="40" spans="1:22" ht="15.75" customHeight="1">
       <c r="A40" s="4" t="s">
         <v>101</v>
       </c>
@@ -10380,23 +10501,26 @@
       <c r="P40" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="Q40" s="4" t="s">
+      <c r="Q40" s="4">
+        <v>990</v>
+      </c>
+      <c r="R40" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="R40" s="4" t="s">
+      <c r="S40" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="S40" s="4" t="b">
+      <c r="T40" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T40" s="4" t="b">
+      <c r="U40" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="U40" s="4" t="s">
+      <c r="V40" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="1:21" ht="15.75" customHeight="1">
+    <row r="41" spans="1:22" ht="15.75" customHeight="1">
       <c r="A41" s="4" t="s">
         <v>101</v>
       </c>
@@ -10445,23 +10569,26 @@
       <c r="P41" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="Q41" s="4" t="s">
+      <c r="Q41" s="4">
+        <v>990</v>
+      </c>
+      <c r="R41" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="R41" s="4" t="s">
+      <c r="S41" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="S41" s="4" t="b">
+      <c r="T41" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T41" s="4" t="b">
+      <c r="U41" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="U41" s="4" t="s">
+      <c r="V41" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="15.75" customHeight="1">
+    <row r="42" spans="1:22" ht="15.75" customHeight="1">
       <c r="A42" s="4" t="s">
         <v>113</v>
       </c>
@@ -10507,20 +10634,23 @@
       <c r="P42" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="Q42" s="4">
+      <c r="Q42" s="35">
+        <v>146</v>
+      </c>
+      <c r="R42" s="4">
         <v>9</v>
       </c>
-      <c r="R42" s="4" t="s">
+      <c r="S42" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="S42" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T42" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U42" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" ht="15.75" customHeight="1">
       <c r="A43" s="35" t="s">
         <v>113</v>
       </c>
@@ -10568,22 +10698,25 @@
         <v>119</v>
       </c>
       <c r="Q43" s="35">
+        <v>146</v>
+      </c>
+      <c r="R43" s="35">
         <v>9</v>
       </c>
-      <c r="R43" s="35" t="s">
+      <c r="S43" s="35" t="s">
         <v>120</v>
-      </c>
-      <c r="S43" s="35" t="b">
-        <v>0</v>
       </c>
       <c r="T43" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="U43" s="40" t="s">
+      <c r="U43" s="35" t="b">
+        <v>0</v>
+      </c>
+      <c r="V43" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="44" spans="1:21" ht="15.75" customHeight="1">
+    <row r="44" spans="1:22" ht="15.75" customHeight="1">
       <c r="A44" s="38" t="s">
         <v>113</v>
       </c>
@@ -10632,23 +10765,26 @@
       <c r="P44" s="38" t="s">
         <v>119</v>
       </c>
-      <c r="Q44" s="38">
+      <c r="Q44" s="35">
+        <v>146</v>
+      </c>
+      <c r="R44" s="38">
         <v>9</v>
       </c>
-      <c r="R44" s="38" t="s">
+      <c r="S44" s="38" t="s">
         <v>150</v>
       </c>
-      <c r="S44" s="35" t="b">
+      <c r="T44" s="35" t="b">
         <v>0</v>
       </c>
-      <c r="T44" s="38" t="b">
+      <c r="U44" s="38" t="b">
         <v>1</v>
       </c>
-      <c r="U44" s="40" t="s">
+      <c r="V44" s="40" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="45" spans="1:21" ht="15.75" customHeight="1">
+    <row r="45" spans="1:22" ht="15.75" customHeight="1">
       <c r="A45" s="4" t="s">
         <v>113</v>
       </c>
@@ -10695,19 +10831,22 @@
         <v>124</v>
       </c>
       <c r="Q45" s="4">
+        <v>17</v>
+      </c>
+      <c r="R45" s="4">
         <v>9</v>
       </c>
-      <c r="R45" s="4" t="s">
+      <c r="S45" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="S45" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T45" s="4" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U45" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" ht="15.75" customHeight="1">
       <c r="A46" s="4" t="s">
         <v>113</v>
       </c>
@@ -10754,22 +10893,25 @@
         <v>124</v>
       </c>
       <c r="Q46" s="4">
+        <v>17</v>
+      </c>
+      <c r="R46" s="4">
         <v>9</v>
       </c>
-      <c r="R46" s="33" t="s">
+      <c r="S46" s="33" t="s">
         <v>125</v>
-      </c>
-      <c r="S46" s="33" t="b">
-        <v>0</v>
       </c>
       <c r="T46" s="33" t="b">
         <v>0</v>
       </c>
-      <c r="U46" s="29" t="s">
+      <c r="U46" s="33" t="b">
+        <v>0</v>
+      </c>
+      <c r="V46" s="29" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="47" spans="1:21" ht="15.75" customHeight="1">
+    <row r="47" spans="1:22" ht="15.75" customHeight="1">
       <c r="A47" s="4" t="s">
         <v>113</v>
       </c>
@@ -10817,19 +10959,22 @@
         <v>124</v>
       </c>
       <c r="Q47" s="4">
+        <v>17</v>
+      </c>
+      <c r="R47" s="4">
         <v>9</v>
       </c>
-      <c r="R47" s="33" t="s">
+      <c r="S47" s="33" t="s">
         <v>52</v>
-      </c>
-      <c r="S47" s="33" t="b">
-        <v>1</v>
       </c>
       <c r="T47" s="33" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U47" s="33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" ht="15.75" customHeight="1">
       <c r="A48" s="4" t="s">
         <v>113</v>
       </c>
@@ -10876,19 +11021,22 @@
         <v>124</v>
       </c>
       <c r="Q48" s="4">
+        <v>17</v>
+      </c>
+      <c r="R48" s="4">
         <v>9</v>
       </c>
-      <c r="R48" s="4" t="s">
+      <c r="S48" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="S48" s="4" t="b">
+      <c r="T48" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T48" s="4" t="b">
+      <c r="U48" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="15.75" customHeight="1">
+    <row r="49" spans="1:22" ht="15.75" customHeight="1">
       <c r="A49" s="11" t="s">
         <v>127</v>
       </c>
@@ -10937,20 +11085,23 @@
       <c r="P49" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q49" s="11" t="s">
+      <c r="Q49" s="12">
+        <v>123</v>
+      </c>
+      <c r="R49" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R49" s="11" t="s">
+      <c r="S49" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="S49" s="4" t="b">
+      <c r="T49" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T49" s="4" t="b">
+      <c r="U49" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="15.75" customHeight="1">
+    <row r="50" spans="1:22" ht="15.75" customHeight="1">
       <c r="A50" s="11" t="s">
         <v>127</v>
       </c>
@@ -10999,20 +11150,23 @@
       <c r="P50" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q50" s="11" t="s">
+      <c r="Q50" s="12">
+        <v>123</v>
+      </c>
+      <c r="R50" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R50" s="11" t="s">
+      <c r="S50" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="S50" s="4" t="b">
+      <c r="T50" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T50" s="4" t="b">
+      <c r="U50" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="15.75" customHeight="1">
+    <row r="51" spans="1:22" ht="15.75" customHeight="1">
       <c r="A51" s="11" t="s">
         <v>127</v>
       </c>
@@ -11061,20 +11215,23 @@
       <c r="P51" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q51" s="11" t="s">
+      <c r="Q51" s="12">
+        <v>123</v>
+      </c>
+      <c r="R51" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R51" s="11" t="s">
+      <c r="S51" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="S51" s="4" t="b">
+      <c r="T51" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T51" s="4" t="b">
+      <c r="U51" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="15.75" customHeight="1">
+    <row r="52" spans="1:22" ht="15.75" customHeight="1">
       <c r="A52" s="11" t="s">
         <v>127</v>
       </c>
@@ -11123,20 +11280,23 @@
       <c r="P52" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q52" s="11" t="s">
+      <c r="Q52" s="12">
+        <v>123</v>
+      </c>
+      <c r="R52" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R52" s="11" t="s">
+      <c r="S52" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="S52" s="4" t="b">
+      <c r="T52" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T52" s="4" t="b">
+      <c r="U52" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="15.75" customHeight="1">
+    <row r="53" spans="1:22" ht="15.75" customHeight="1">
       <c r="A53" s="11" t="s">
         <v>127</v>
       </c>
@@ -11185,23 +11345,26 @@
       <c r="P53" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q53" s="11" t="s">
+      <c r="Q53" s="12">
+        <v>123</v>
+      </c>
+      <c r="R53" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R53" s="11" t="s">
+      <c r="S53" s="11" t="s">
         <v>137</v>
-      </c>
-      <c r="S53" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T53" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="U53" s="11" t="s">
+      <c r="U53" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="V53" s="11" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="15.75" customHeight="1">
+    <row r="54" spans="1:22" ht="15.75" customHeight="1">
       <c r="A54" s="11" t="s">
         <v>127</v>
       </c>
@@ -11250,23 +11413,26 @@
       <c r="P54" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q54" s="11" t="s">
+      <c r="Q54" s="12">
+        <v>123</v>
+      </c>
+      <c r="R54" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R54" s="11" t="s">
+      <c r="S54" s="11" t="s">
         <v>138</v>
-      </c>
-      <c r="S54" s="4" t="b">
-        <v>0</v>
       </c>
       <c r="T54" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="U54" s="11" t="s">
+      <c r="U54" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="V54" s="11" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="15.75" customHeight="1">
+    <row r="55" spans="1:22" ht="15.75" customHeight="1">
       <c r="A55" s="11" t="s">
         <v>127</v>
       </c>
@@ -11317,21 +11483,24 @@
       <c r="P55" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q55" s="11" t="s">
+      <c r="Q55" s="12">
+        <v>123</v>
+      </c>
+      <c r="R55" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R55" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="S55" s="4" t="b">
-        <v>1</v>
+      <c r="S55" s="11" t="s">
+        <v>205</v>
       </c>
       <c r="T55" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="U55" s="11"/>
-    </row>
-    <row r="56" spans="1:21" ht="15.75" customHeight="1">
+      <c r="U55" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="V55" s="11"/>
+    </row>
+    <row r="56" spans="1:22" ht="15.75" customHeight="1">
       <c r="A56" s="11" t="s">
         <v>127</v>
       </c>
@@ -11380,48 +11549,51 @@
       <c r="P56" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="Q56" s="11" t="s">
+      <c r="Q56" s="12">
+        <v>123</v>
+      </c>
+      <c r="R56" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="R56" s="11" t="s">
+      <c r="S56" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="S56" s="4" t="b">
+      <c r="T56" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="T56" s="4" t="b">
+      <c r="U56" s="4" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="15.75" customHeight="1">
+    <row r="57" spans="1:22" ht="15.75" customHeight="1">
       <c r="F57" s="5"/>
       <c r="J57" s="5"/>
     </row>
-    <row r="58" spans="1:21" ht="15.75" customHeight="1">
+    <row r="58" spans="1:22" ht="15.75" customHeight="1">
       <c r="F58" s="5"/>
       <c r="J58" s="5"/>
     </row>
-    <row r="59" spans="1:21" ht="15.75" customHeight="1">
+    <row r="59" spans="1:22" ht="15.75" customHeight="1">
       <c r="F59" s="5"/>
       <c r="J59" s="5"/>
     </row>
-    <row r="60" spans="1:21" ht="15.75" customHeight="1">
+    <row r="60" spans="1:22" ht="15.75" customHeight="1">
       <c r="F60" s="5"/>
       <c r="J60" s="5"/>
     </row>
-    <row r="61" spans="1:21" ht="15.75" customHeight="1">
+    <row r="61" spans="1:22" ht="15.75" customHeight="1">
       <c r="F61" s="5"/>
       <c r="J61" s="5"/>
     </row>
-    <row r="62" spans="1:21" ht="15.75" customHeight="1">
+    <row r="62" spans="1:22" ht="15.75" customHeight="1">
       <c r="F62" s="5"/>
       <c r="J62" s="5"/>
     </row>
-    <row r="63" spans="1:21" ht="15.75" customHeight="1">
+    <row r="63" spans="1:22" ht="15.75" customHeight="1">
       <c r="F63" s="5"/>
       <c r="J63" s="5"/>
     </row>
-    <row r="64" spans="1:21" ht="15.75" customHeight="1">
+    <row r="64" spans="1:22" ht="15.75" customHeight="1">
       <c r="F64" s="5"/>
       <c r="J64" s="5"/>
     </row>
@@ -15206,7 +15378,7 @@
       <c r="J1009" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="S1:S1009" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="T1:T1009" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="M55:N55" formulaRange="1"/>

</xml_diff>

<commit_message>
minor edits to data
</commit_message>
<xml_diff>
--- a/data/sar_extraction.xlsx
+++ b/data/sar_extraction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ginacuomo-dannenburg/Documents/code/bvd-contacts/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E35BB9-B215-B24A-85E1-4E19F01D9950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B0A36B-1BA2-8541-AE93-71F5176DB656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25520" yWindow="-12140" windowWidth="25360" windowHeight="27180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_extraction" sheetId="1" r:id="rId1"/>
@@ -908,7 +908,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -984,12 +984,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -1086,7 +1080,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1148,12 +1142,7 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1164,22 +1153,16 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -7984,7 +7967,6 @@
     <col min="18" max="18" width="15.6640625" customWidth="1"/>
     <col min="19" max="19" width="51" customWidth="1"/>
     <col min="22" max="22" width="112.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="12.6640625" style="42"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="16">
@@ -8054,12 +8036,12 @@
       <c r="V1" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="W1" s="41"/>
-      <c r="X1" s="41"/>
-      <c r="Y1" s="41"/>
-      <c r="Z1" s="41"/>
-      <c r="AA1" s="41"/>
-      <c r="AB1" s="41"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
+      <c r="AA1" s="3"/>
+      <c r="AB1" s="3"/>
     </row>
     <row r="2" spans="1:28" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
@@ -9570,478 +9552,478 @@
       </c>
     </row>
     <row r="25" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A25" s="35" t="s">
+      <c r="A25" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B25" s="35">
+      <c r="B25" s="32">
         <v>2003</v>
       </c>
-      <c r="C25" s="35" t="s">
+      <c r="C25" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D25" s="35" t="s">
+      <c r="D25" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E25" s="35" t="s">
+      <c r="E25" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F25" s="36" t="s">
+      <c r="F25" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G25" s="35" t="s">
+      <c r="G25" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H25" s="35" t="s">
+      <c r="H25" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I25" s="35" t="s">
+      <c r="I25" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="J25" s="36">
+      <c r="J25" s="33">
         <v>9</v>
       </c>
-      <c r="K25" s="35">
+      <c r="K25" s="32">
         <v>2</v>
       </c>
-      <c r="L25" s="35">
+      <c r="L25" s="32">
         <v>9</v>
       </c>
-      <c r="M25" s="35">
+      <c r="M25" s="32">
         <v>24</v>
       </c>
-      <c r="N25" s="35">
+      <c r="N25" s="32">
         <v>89</v>
       </c>
-      <c r="O25" s="35">
+      <c r="O25" s="32">
         <v>89</v>
       </c>
-      <c r="P25" s="35" t="s">
+      <c r="P25" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q25" s="35">
+      <c r="Q25" s="32">
         <v>27</v>
       </c>
-      <c r="R25" s="35">
+      <c r="R25" s="32">
         <v>9</v>
       </c>
-      <c r="S25" s="35" t="s">
+      <c r="S25" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="T25" s="35" t="b">
+      <c r="T25" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U25" s="35" t="b">
+      <c r="U25" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V25" s="40" t="s">
+      <c r="V25" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A26" s="35" t="s">
+      <c r="A26" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B26" s="35">
+      <c r="B26" s="32">
         <v>2003</v>
       </c>
-      <c r="C26" s="35" t="s">
+      <c r="C26" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D26" s="35" t="s">
+      <c r="D26" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="35" t="s">
+      <c r="E26" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="36" t="s">
+      <c r="F26" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G26" s="35" t="s">
+      <c r="G26" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H26" s="35" t="s">
+      <c r="H26" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I26" s="35" t="s">
+      <c r="I26" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="J26" s="36">
+      <c r="J26" s="33">
         <v>9</v>
       </c>
-      <c r="K26" s="35">
+      <c r="K26" s="32">
         <v>2</v>
       </c>
-      <c r="L26" s="35">
+      <c r="L26" s="32">
         <v>9</v>
       </c>
-      <c r="M26" s="35">
+      <c r="M26" s="32">
         <v>19</v>
       </c>
-      <c r="N26" s="35">
+      <c r="N26" s="32">
         <v>70</v>
       </c>
-      <c r="O26" s="35">
+      <c r="O26" s="32">
         <v>89</v>
       </c>
-      <c r="P26" s="35" t="s">
+      <c r="P26" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q26" s="35">
+      <c r="Q26" s="32">
         <v>27</v>
       </c>
-      <c r="R26" s="35">
+      <c r="R26" s="32">
         <v>9</v>
       </c>
-      <c r="S26" s="35" t="s">
+      <c r="S26" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="T26" s="35" t="b">
+      <c r="T26" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U26" s="35" t="b">
+      <c r="U26" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V26" s="40" t="s">
+      <c r="V26" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B27" s="35">
+      <c r="B27" s="32">
         <v>2003</v>
       </c>
-      <c r="C27" s="35" t="s">
+      <c r="C27" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="35" t="s">
+      <c r="D27" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="35" t="s">
+      <c r="E27" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F27" s="36" t="s">
+      <c r="F27" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G27" s="35" t="s">
+      <c r="G27" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H27" s="35" t="s">
+      <c r="H27" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I27" s="35" t="s">
+      <c r="I27" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="J27" s="36">
+      <c r="J27" s="33">
         <v>9</v>
       </c>
-      <c r="K27" s="35">
+      <c r="K27" s="32">
         <v>2</v>
       </c>
-      <c r="L27" s="35">
+      <c r="L27" s="32">
         <v>9</v>
       </c>
-      <c r="M27" s="35">
+      <c r="M27" s="32">
         <v>1</v>
       </c>
-      <c r="N27" s="35">
+      <c r="N27" s="32">
         <v>13</v>
       </c>
-      <c r="O27" s="35">
+      <c r="O27" s="32">
         <v>89</v>
       </c>
-      <c r="P27" s="35" t="s">
+      <c r="P27" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q27" s="35">
+      <c r="Q27" s="32">
         <v>27</v>
       </c>
-      <c r="R27" s="35">
+      <c r="R27" s="32">
         <v>9</v>
       </c>
-      <c r="S27" s="35" t="s">
+      <c r="S27" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="T27" s="35" t="b">
+      <c r="T27" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U27" s="35" t="b">
+      <c r="U27" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V27" s="40" t="s">
+      <c r="V27" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A28" s="35" t="s">
+      <c r="A28" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="35">
+      <c r="B28" s="32">
         <v>2003</v>
       </c>
-      <c r="C28" s="35" t="s">
+      <c r="C28" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D28" s="35" t="s">
+      <c r="D28" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E28" s="35" t="s">
+      <c r="E28" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F28" s="36" t="s">
+      <c r="F28" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G28" s="35" t="s">
+      <c r="G28" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H28" s="35" t="s">
+      <c r="H28" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I28" s="35" t="s">
+      <c r="I28" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="J28" s="36">
+      <c r="J28" s="33">
         <v>9</v>
       </c>
-      <c r="K28" s="35">
+      <c r="K28" s="32">
         <v>2</v>
       </c>
-      <c r="L28" s="35">
+      <c r="L28" s="32">
         <v>9</v>
       </c>
-      <c r="M28" s="35">
+      <c r="M28" s="32">
         <v>15</v>
       </c>
-      <c r="N28" s="35">
+      <c r="N28" s="32">
         <v>30</v>
       </c>
-      <c r="O28" s="35">
+      <c r="O28" s="32">
         <v>89</v>
       </c>
-      <c r="P28" s="35" t="s">
+      <c r="P28" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q28" s="35">
+      <c r="Q28" s="32">
         <v>27</v>
       </c>
-      <c r="R28" s="35">
+      <c r="R28" s="32">
         <v>9</v>
       </c>
-      <c r="S28" s="35" t="s">
+      <c r="S28" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="T28" s="35" t="b">
+      <c r="T28" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U28" s="35" t="b">
+      <c r="U28" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V28" s="40" t="s">
+      <c r="V28" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="29" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A29" s="35" t="s">
+      <c r="A29" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="35">
+      <c r="B29" s="32">
         <v>2003</v>
       </c>
-      <c r="C29" s="35" t="s">
+      <c r="C29" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D29" s="35" t="s">
+      <c r="D29" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E29" s="35" t="s">
+      <c r="E29" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F29" s="36" t="s">
+      <c r="F29" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G29" s="35" t="s">
+      <c r="G29" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H29" s="35" t="s">
+      <c r="H29" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I29" s="35" t="s">
+      <c r="I29" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="J29" s="36">
+      <c r="J29" s="33">
         <v>9</v>
       </c>
-      <c r="K29" s="35">
+      <c r="K29" s="32">
         <v>2</v>
       </c>
-      <c r="L29" s="35">
+      <c r="L29" s="32">
         <v>9</v>
       </c>
-      <c r="M29" s="35">
+      <c r="M29" s="32">
         <v>5</v>
       </c>
-      <c r="N29" s="35">
+      <c r="N29" s="32">
         <v>53</v>
       </c>
-      <c r="O29" s="35">
+      <c r="O29" s="32">
         <v>89</v>
       </c>
-      <c r="P29" s="35" t="s">
+      <c r="P29" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q29" s="35">
+      <c r="Q29" s="32">
         <v>27</v>
       </c>
-      <c r="R29" s="35">
+      <c r="R29" s="32">
         <v>9</v>
       </c>
-      <c r="S29" s="35" t="s">
+      <c r="S29" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="T29" s="35" t="b">
+      <c r="T29" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U29" s="35" t="b">
+      <c r="U29" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V29" s="40" t="s">
+      <c r="V29" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="30" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A30" s="35" t="s">
+      <c r="A30" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B30" s="35">
+      <c r="B30" s="32">
         <v>2003</v>
       </c>
-      <c r="C30" s="35" t="s">
+      <c r="C30" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="35" t="s">
+      <c r="D30" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E30" s="35" t="s">
+      <c r="E30" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F30" s="36" t="s">
+      <c r="F30" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G30" s="35" t="s">
+      <c r="G30" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H30" s="35" t="s">
+      <c r="H30" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I30" s="35" t="s">
+      <c r="I30" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="J30" s="36">
+      <c r="J30" s="33">
         <v>9</v>
       </c>
-      <c r="K30" s="35">
+      <c r="K30" s="32">
         <v>2</v>
       </c>
-      <c r="L30" s="35">
+      <c r="L30" s="32">
         <v>9</v>
       </c>
-      <c r="M30" s="35">
+      <c r="M30" s="32">
         <v>2</v>
       </c>
-      <c r="N30" s="35">
+      <c r="N30" s="32">
         <v>40</v>
       </c>
-      <c r="O30" s="35">
+      <c r="O30" s="32">
         <v>89</v>
       </c>
-      <c r="P30" s="35" t="s">
+      <c r="P30" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q30" s="35">
+      <c r="Q30" s="32">
         <v>27</v>
       </c>
-      <c r="R30" s="35">
+      <c r="R30" s="32">
         <v>9</v>
       </c>
-      <c r="S30" s="35" t="s">
+      <c r="S30" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="T30" s="35" t="b">
+      <c r="T30" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U30" s="35" t="b">
+      <c r="U30" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V30" s="40" t="s">
+      <c r="V30" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A31" s="35" t="s">
+      <c r="A31" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="35">
+      <c r="B31" s="32">
         <v>2003</v>
       </c>
-      <c r="C31" s="35" t="s">
+      <c r="C31" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D31" s="35" t="s">
+      <c r="D31" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E31" s="35" t="s">
+      <c r="E31" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F31" s="36" t="s">
+      <c r="F31" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G31" s="35" t="s">
+      <c r="G31" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H31" s="35" t="s">
+      <c r="H31" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I31" s="35" t="s">
+      <c r="I31" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="J31" s="36">
+      <c r="J31" s="33">
         <v>9</v>
       </c>
-      <c r="K31" s="35">
+      <c r="K31" s="32">
         <v>2</v>
       </c>
-      <c r="L31" s="35">
+      <c r="L31" s="32">
         <v>9</v>
       </c>
-      <c r="M31" s="35">
+      <c r="M31" s="32">
         <v>18</v>
       </c>
-      <c r="N31" s="35">
+      <c r="N31" s="32">
         <v>43</v>
       </c>
-      <c r="O31" s="35">
+      <c r="O31" s="32">
         <v>89</v>
       </c>
-      <c r="P31" s="35" t="s">
+      <c r="P31" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q31" s="35">
+      <c r="Q31" s="32">
         <v>27</v>
       </c>
-      <c r="R31" s="35">
+      <c r="R31" s="32">
         <v>9</v>
       </c>
-      <c r="S31" s="35" t="s">
+      <c r="S31" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="T31" s="35" t="b">
+      <c r="T31" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U31" s="35" t="b">
+      <c r="U31" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V31" s="40" t="s">
+      <c r="V31" s="37" t="s">
         <v>202</v>
       </c>
     </row>
@@ -10756,7 +10738,7 @@
       <c r="P42" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="Q42" s="35">
+      <c r="Q42" s="32">
         <v>146</v>
       </c>
       <c r="R42" s="4">
@@ -10773,136 +10755,136 @@
       </c>
     </row>
     <row r="43" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A43" s="35" t="s">
+      <c r="A43" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="B43" s="35">
+      <c r="B43" s="32">
         <v>1978</v>
       </c>
-      <c r="C43" s="35" t="s">
+      <c r="C43" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="D43" s="35" t="s">
+      <c r="D43" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="E43" s="35" t="s">
+      <c r="E43" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="F43" s="36">
+      <c r="F43" s="33">
         <v>1976</v>
       </c>
-      <c r="G43" s="37"/>
-      <c r="H43" s="35" t="s">
+      <c r="G43" s="34"/>
+      <c r="H43" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="I43" s="35" t="s">
+      <c r="I43" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="J43" s="36" t="s">
+      <c r="J43" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="K43" s="35">
+      <c r="K43" s="32">
         <v>1</v>
       </c>
-      <c r="L43" s="35" t="s">
+      <c r="L43" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="M43" s="35">
+      <c r="M43" s="32">
         <v>37</v>
       </c>
-      <c r="N43" s="35">
+      <c r="N43" s="32">
         <v>135</v>
       </c>
-      <c r="O43" s="35">
+      <c r="O43" s="32">
         <v>1103</v>
       </c>
-      <c r="P43" s="35" t="s">
+      <c r="P43" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="Q43" s="35">
+      <c r="Q43" s="32">
         <v>146</v>
       </c>
-      <c r="R43" s="35">
+      <c r="R43" s="32">
         <v>9</v>
       </c>
-      <c r="S43" s="35" t="s">
+      <c r="S43" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="T43" s="35" t="b">
+      <c r="T43" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U43" s="35" t="b">
+      <c r="U43" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V43" s="40" t="s">
+      <c r="V43" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="44" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A44" s="38" t="s">
+      <c r="A44" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="B44" s="38">
+      <c r="B44" s="35">
         <v>1978</v>
       </c>
-      <c r="C44" s="38" t="s">
+      <c r="C44" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="D44" s="38" t="s">
+      <c r="D44" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="E44" s="38" t="s">
+      <c r="E44" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="F44" s="39">
+      <c r="F44" s="36">
         <v>1976</v>
       </c>
-      <c r="G44" s="38"/>
-      <c r="H44" s="38" t="s">
+      <c r="G44" s="35"/>
+      <c r="H44" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="I44" s="38" t="s">
+      <c r="I44" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="J44" s="39" t="s">
+      <c r="J44" s="36" t="s">
         <v>149</v>
       </c>
-      <c r="K44" s="38">
+      <c r="K44" s="35">
         <v>1</v>
       </c>
-      <c r="L44" s="38" t="s">
+      <c r="L44" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="M44" s="38">
+      <c r="M44" s="35">
         <f>M42-M43</f>
         <v>25</v>
       </c>
-      <c r="N44" s="38">
+      <c r="N44" s="35">
         <f>O43-N43</f>
         <v>968</v>
       </c>
-      <c r="O44" s="38">
+      <c r="O44" s="35">
         <v>1103</v>
       </c>
-      <c r="P44" s="38" t="s">
+      <c r="P44" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="Q44" s="35">
+      <c r="Q44" s="32">
         <v>146</v>
       </c>
-      <c r="R44" s="38">
+      <c r="R44" s="35">
         <v>9</v>
       </c>
-      <c r="S44" s="38" t="s">
+      <c r="S44" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="T44" s="35" t="b">
+      <c r="T44" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U44" s="38" t="b">
+      <c r="U44" s="35" t="b">
         <v>1</v>
       </c>
-      <c r="V44" s="40" t="s">
+      <c r="V44" s="37" t="s">
         <v>202</v>
       </c>
     </row>
@@ -11020,13 +11002,13 @@
       <c r="R46" s="4">
         <v>9</v>
       </c>
-      <c r="S46" s="33" t="s">
+      <c r="S46" s="31" t="s">
         <v>125</v>
       </c>
-      <c r="T46" s="33" t="b">
+      <c r="T46" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="U46" s="33" t="b">
+      <c r="U46" s="31" t="b">
         <v>0</v>
       </c>
       <c r="V46" s="29" t="s">
@@ -11086,13 +11068,13 @@
       <c r="R47" s="4">
         <v>9</v>
       </c>
-      <c r="S47" s="33" t="s">
+      <c r="S47" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="T47" s="33" t="b">
+      <c r="T47" s="31" t="b">
         <v>1</v>
       </c>
-      <c r="U47" s="33" t="b">
+      <c r="U47" s="31" t="b">
         <v>1</v>
       </c>
     </row>
@@ -15520,10 +15502,9 @@
     <col min="12" max="12" width="21.1640625" customWidth="1"/>
     <col min="15" max="15" width="14.5" customWidth="1"/>
     <col min="16" max="17" width="15.5" customWidth="1"/>
-    <col min="18" max="18" width="15.6640625" style="42" customWidth="1"/>
+    <col min="18" max="18" width="15.6640625" customWidth="1"/>
     <col min="19" max="19" width="51" customWidth="1"/>
     <col min="22" max="22" width="112.6640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="12.6640625" style="42"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="16">
@@ -15578,7 +15559,7 @@
       <c r="Q1" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="R1" s="45" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="S1" s="13" t="s">
@@ -15593,12 +15574,12 @@
       <c r="V1" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="W1" s="41"/>
-      <c r="X1" s="41"/>
-      <c r="Y1" s="41"/>
-      <c r="Z1" s="41"/>
-      <c r="AA1" s="41"/>
-      <c r="AB1" s="41"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
+      <c r="AA1" s="3"/>
+      <c r="AB1" s="3"/>
     </row>
     <row r="2" spans="1:28" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
@@ -15652,7 +15633,7 @@
       <c r="Q2" s="4">
         <v>34</v>
       </c>
-      <c r="R2" s="46">
+      <c r="R2" s="4">
         <v>9</v>
       </c>
       <c r="S2" s="4" t="s">
@@ -15717,7 +15698,7 @@
       <c r="Q3" s="4">
         <v>34</v>
       </c>
-      <c r="R3" s="46">
+      <c r="R3" s="4">
         <v>9</v>
       </c>
       <c r="S3" s="4" t="s">
@@ -15782,7 +15763,7 @@
       <c r="Q4" s="4">
         <v>34</v>
       </c>
-      <c r="R4" s="46">
+      <c r="R4" s="4">
         <v>9</v>
       </c>
       <c r="S4" s="4" t="s">
@@ -15847,7 +15828,7 @@
       <c r="Q5" s="4">
         <v>34</v>
       </c>
-      <c r="R5" s="46">
+      <c r="R5" s="4">
         <v>9</v>
       </c>
       <c r="S5" s="4" t="s">
@@ -15912,7 +15893,7 @@
       <c r="Q6" s="4">
         <v>34</v>
       </c>
-      <c r="R6" s="46">
+      <c r="R6" s="4">
         <v>9</v>
       </c>
       <c r="S6" s="4" t="s">
@@ -15978,7 +15959,7 @@
         <f>117+27</f>
         <v>144</v>
       </c>
-      <c r="R7" s="46">
+      <c r="R7" s="4">
         <v>9</v>
       </c>
       <c r="S7" s="4" t="s">
@@ -16043,7 +16024,7 @@
       <c r="Q8" s="4">
         <v>144</v>
       </c>
-      <c r="R8" s="46">
+      <c r="R8" s="4">
         <v>9</v>
       </c>
       <c r="S8" s="4" t="s">
@@ -16108,7 +16089,7 @@
       <c r="Q9" s="4">
         <v>144</v>
       </c>
-      <c r="R9" s="46">
+      <c r="R9" s="4">
         <v>9</v>
       </c>
       <c r="S9" s="4" t="s">
@@ -16173,7 +16154,7 @@
       <c r="Q10" s="4">
         <v>30</v>
       </c>
-      <c r="R10" s="46">
+      <c r="R10" s="4">
         <v>9</v>
       </c>
       <c r="S10" s="4" t="s">
@@ -16223,10 +16204,10 @@
       <c r="L11" s="4">
         <v>9</v>
       </c>
-      <c r="M11" s="44">
+      <c r="M11" s="39">
         <v>19</v>
       </c>
-      <c r="N11" s="44">
+      <c r="N11" s="39">
         <v>137</v>
       </c>
       <c r="O11" s="4">
@@ -16238,7 +16219,7 @@
       <c r="Q11" s="4">
         <v>30</v>
       </c>
-      <c r="R11" s="46">
+      <c r="R11" s="4">
         <v>9</v>
       </c>
       <c r="S11" s="4" t="s">
@@ -16303,7 +16284,7 @@
       <c r="Q12" s="4">
         <v>30</v>
       </c>
-      <c r="R12" s="46">
+      <c r="R12" s="4">
         <v>9</v>
       </c>
       <c r="S12" s="4" t="s">
@@ -16316,7 +16297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="50" customFormat="1" ht="15.75" customHeight="1">
+    <row r="13" spans="1:28" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>54</v>
       </c>
@@ -16332,7 +16313,7 @@
       <c r="E13" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="48" t="s">
+      <c r="F13" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -16344,7 +16325,7 @@
       <c r="I13" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J13" s="49">
+      <c r="J13" s="41">
         <v>9</v>
       </c>
       <c r="K13" s="3">
@@ -16368,7 +16349,7 @@
       <c r="Q13" s="3">
         <v>150</v>
       </c>
-      <c r="R13" s="41">
+      <c r="R13" s="3">
         <v>9</v>
       </c>
       <c r="S13" s="3" t="s">
@@ -16380,9 +16361,8 @@
       <c r="U13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V13" s="30"/>
-    </row>
-    <row r="14" spans="1:28" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="14" spans="1:28" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>54</v>
       </c>
@@ -16398,7 +16378,7 @@
       <c r="E14" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="48" t="s">
+      <c r="F14" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G14" s="3" t="s">
@@ -16410,7 +16390,7 @@
       <c r="I14" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="J14" s="49">
+      <c r="J14" s="41">
         <v>9</v>
       </c>
       <c r="K14" s="3">
@@ -16434,7 +16414,7 @@
       <c r="Q14" s="3">
         <v>150</v>
       </c>
-      <c r="R14" s="41">
+      <c r="R14" s="3">
         <v>9</v>
       </c>
       <c r="S14" s="3" t="s">
@@ -16446,9 +16426,8 @@
       <c r="U14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V14" s="30"/>
-    </row>
-    <row r="15" spans="1:28" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="15" spans="1:28" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A15" s="3" t="s">
         <v>54</v>
       </c>
@@ -16464,7 +16443,7 @@
       <c r="E15" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="48" t="s">
+      <c r="F15" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -16476,7 +16455,7 @@
       <c r="I15" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="J15" s="49">
+      <c r="J15" s="41">
         <v>9</v>
       </c>
       <c r="K15" s="3">
@@ -16500,7 +16479,7 @@
       <c r="Q15" s="3">
         <v>150</v>
       </c>
-      <c r="R15" s="41">
+      <c r="R15" s="3">
         <v>9</v>
       </c>
       <c r="S15" s="3" t="s">
@@ -16512,9 +16491,8 @@
       <c r="U15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V15" s="30"/>
-    </row>
-    <row r="16" spans="1:28" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="16" spans="1:28" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A16" s="3" t="s">
         <v>54</v>
       </c>
@@ -16530,7 +16508,7 @@
       <c r="E16" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F16" s="48" t="s">
+      <c r="F16" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G16" s="3" t="s">
@@ -16542,7 +16520,7 @@
       <c r="I16" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="J16" s="49">
+      <c r="J16" s="41">
         <v>9</v>
       </c>
       <c r="K16" s="3">
@@ -16566,7 +16544,7 @@
       <c r="Q16" s="3">
         <v>150</v>
       </c>
-      <c r="R16" s="41">
+      <c r="R16" s="3">
         <v>9</v>
       </c>
       <c r="S16" s="3" t="s">
@@ -16578,9 +16556,8 @@
       <c r="U16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V16" s="30"/>
-    </row>
-    <row r="17" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="17" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>54</v>
       </c>
@@ -16596,7 +16573,7 @@
       <c r="E17" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F17" s="48" t="s">
+      <c r="F17" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -16608,7 +16585,7 @@
       <c r="I17" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="J17" s="49">
+      <c r="J17" s="41">
         <v>9</v>
       </c>
       <c r="K17" s="3">
@@ -16632,7 +16609,7 @@
       <c r="Q17" s="3">
         <v>150</v>
       </c>
-      <c r="R17" s="41">
+      <c r="R17" s="3">
         <v>9</v>
       </c>
       <c r="S17" s="3" t="s">
@@ -16644,9 +16621,8 @@
       <c r="U17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V17" s="30"/>
-    </row>
-    <row r="18" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="18" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A18" s="3" t="s">
         <v>54</v>
       </c>
@@ -16662,7 +16638,7 @@
       <c r="E18" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F18" s="48" t="s">
+      <c r="F18" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G18" s="3" t="s">
@@ -16674,7 +16650,7 @@
       <c r="I18" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="J18" s="49">
+      <c r="J18" s="41">
         <v>9</v>
       </c>
       <c r="K18" s="3">
@@ -16698,7 +16674,7 @@
       <c r="Q18" s="3">
         <v>150</v>
       </c>
-      <c r="R18" s="41">
+      <c r="R18" s="3">
         <v>9</v>
       </c>
       <c r="S18" s="3" t="s">
@@ -16710,9 +16686,8 @@
       <c r="U18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V18" s="30"/>
-    </row>
-    <row r="19" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="19" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A19" s="29" t="s">
         <v>54</v>
       </c>
@@ -16728,7 +16703,7 @@
       <c r="E19" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="F19" s="53" t="s">
+      <c r="F19" s="44" t="s">
         <v>58</v>
       </c>
       <c r="G19" s="29" t="s">
@@ -16764,7 +16739,7 @@
       <c r="Q19" s="29">
         <v>9</v>
       </c>
-      <c r="R19" s="41">
+      <c r="R19" s="3">
         <v>9</v>
       </c>
       <c r="S19" s="3" t="s">
@@ -16772,9 +16747,8 @@
       </c>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
-      <c r="V19" s="30"/>
-    </row>
-    <row r="20" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="20" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A20" s="29" t="s">
         <v>54</v>
       </c>
@@ -16790,7 +16764,7 @@
       <c r="E20" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="F20" s="53" t="s">
+      <c r="F20" s="44" t="s">
         <v>58</v>
       </c>
       <c r="G20" s="29" t="s">
@@ -16826,7 +16800,7 @@
       <c r="Q20" s="29">
         <v>9</v>
       </c>
-      <c r="R20" s="41">
+      <c r="R20" s="3">
         <v>9</v>
       </c>
       <c r="S20" s="3" t="s">
@@ -16834,9 +16808,8 @@
       </c>
       <c r="T20" s="3"/>
       <c r="U20" s="3"/>
-      <c r="V20" s="30"/>
-    </row>
-    <row r="21" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="21" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>54</v>
       </c>
@@ -16852,7 +16825,7 @@
       <c r="E21" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F21" s="48" t="s">
+      <c r="F21" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G21" s="3" t="s">
@@ -16864,7 +16837,7 @@
       <c r="I21" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J21" s="49">
+      <c r="J21" s="41">
         <v>9</v>
       </c>
       <c r="K21" s="3">
@@ -16888,7 +16861,7 @@
       <c r="Q21" s="3">
         <v>150</v>
       </c>
-      <c r="R21" s="41">
+      <c r="R21" s="3">
         <v>9</v>
       </c>
       <c r="S21" s="3" t="s">
@@ -16900,9 +16873,8 @@
       <c r="U21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V21" s="30"/>
-    </row>
-    <row r="22" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
+    </row>
+    <row r="22" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="s">
         <v>54</v>
       </c>
@@ -16918,7 +16890,7 @@
       <c r="E22" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F22" s="48" t="s">
+      <c r="F22" s="40" t="s">
         <v>58</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -16930,7 +16902,7 @@
       <c r="I22" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="J22" s="49">
+      <c r="J22" s="41">
         <v>9</v>
       </c>
       <c r="K22" s="3">
@@ -16954,7 +16926,7 @@
       <c r="Q22" s="3">
         <v>150</v>
       </c>
-      <c r="R22" s="41">
+      <c r="R22" s="3">
         <v>9</v>
       </c>
       <c r="S22" s="3" t="s">
@@ -16966,1913 +16938,1892 @@
       <c r="U22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="V22" s="30"/>
-    </row>
-    <row r="23" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A23" s="54" t="s">
+    </row>
+    <row r="23" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A23" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="54">
+      <c r="B23" s="45">
         <v>2018</v>
       </c>
-      <c r="C23" s="54" t="s">
+      <c r="C23" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="54" t="s">
+      <c r="D23" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E23" s="54" t="s">
+      <c r="E23" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F23" s="54" t="s">
+      <c r="F23" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G23" s="54" t="s">
+      <c r="G23" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H23" s="54" t="s">
+      <c r="H23" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I23" s="54" t="s">
+      <c r="I23" s="45" t="s">
         <v>211</v>
       </c>
-      <c r="J23" s="54">
+      <c r="J23" s="45">
         <v>9</v>
       </c>
-      <c r="K23" s="54">
+      <c r="K23" s="45">
         <v>1</v>
       </c>
-      <c r="L23" s="54" t="s">
+      <c r="L23" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M23" s="54">
+      <c r="M23" s="45">
         <v>38</v>
       </c>
-      <c r="N23" s="54">
+      <c r="N23" s="45">
         <v>222</v>
       </c>
-      <c r="O23" s="54">
+      <c r="O23" s="45">
         <v>838</v>
       </c>
-      <c r="P23" s="54" t="s">
+      <c r="P23" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q23" s="54">
+      <c r="Q23" s="45">
         <v>9</v>
       </c>
-      <c r="R23" s="41"/>
+      <c r="R23" s="3"/>
       <c r="S23" s="3"/>
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
-      <c r="V23" s="30"/>
-    </row>
-    <row r="24" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A24" s="54" t="s">
+    </row>
+    <row r="24" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A24" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="54">
+      <c r="B24" s="45">
         <v>2018</v>
       </c>
-      <c r="C24" s="54" t="s">
+      <c r="C24" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D24" s="54" t="s">
+      <c r="D24" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="54" t="s">
+      <c r="E24" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F24" s="54" t="s">
+      <c r="F24" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G24" s="54" t="s">
+      <c r="G24" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H24" s="54" t="s">
+      <c r="H24" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I24" s="54" t="s">
+      <c r="I24" s="45" t="s">
         <v>212</v>
       </c>
-      <c r="J24" s="54">
+      <c r="J24" s="45">
         <v>9</v>
       </c>
-      <c r="K24" s="54">
+      <c r="K24" s="45">
         <v>1</v>
       </c>
-      <c r="L24" s="54" t="s">
+      <c r="L24" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M24" s="54">
+      <c r="M24" s="45">
         <v>45</v>
       </c>
-      <c r="N24" s="54">
+      <c r="N24" s="45">
         <v>616</v>
       </c>
-      <c r="O24" s="54">
+      <c r="O24" s="45">
         <v>838</v>
       </c>
-      <c r="P24" s="54" t="s">
+      <c r="P24" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q24" s="54">
+      <c r="Q24" s="45">
         <v>9</v>
       </c>
-      <c r="R24" s="41"/>
+      <c r="R24" s="3"/>
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
-      <c r="V24" s="30"/>
-    </row>
-    <row r="25" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A25" s="54" t="s">
+    </row>
+    <row r="25" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A25" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="54">
+      <c r="B25" s="45">
         <v>2018</v>
       </c>
-      <c r="C25" s="54" t="s">
+      <c r="C25" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D25" s="54" t="s">
+      <c r="D25" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="54" t="s">
+      <c r="E25" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F25" s="54" t="s">
+      <c r="F25" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G25" s="54" t="s">
+      <c r="G25" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H25" s="54" t="s">
+      <c r="H25" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I25" s="54" t="s">
+      <c r="I25" s="45" t="s">
         <v>213</v>
       </c>
-      <c r="J25" s="54">
+      <c r="J25" s="45">
         <v>9</v>
       </c>
-      <c r="K25" s="54">
+      <c r="K25" s="45">
         <v>1</v>
       </c>
-      <c r="L25" s="54" t="s">
+      <c r="L25" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M25" s="54">
+      <c r="M25" s="45">
         <v>32</v>
       </c>
-      <c r="N25" s="54">
+      <c r="N25" s="45">
         <v>216</v>
       </c>
-      <c r="O25" s="54">
+      <c r="O25" s="45">
         <v>838</v>
       </c>
-      <c r="P25" s="54" t="s">
+      <c r="P25" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q25" s="54">
+      <c r="Q25" s="45">
         <v>9</v>
       </c>
-      <c r="R25" s="41"/>
+      <c r="R25" s="3"/>
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
-      <c r="V25" s="30"/>
-    </row>
-    <row r="26" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A26" s="54" t="s">
+    </row>
+    <row r="26" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A26" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="54">
+      <c r="B26" s="45">
         <v>2018</v>
       </c>
-      <c r="C26" s="54" t="s">
+      <c r="C26" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="54" t="s">
+      <c r="D26" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="54" t="s">
+      <c r="E26" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="54" t="s">
+      <c r="F26" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G26" s="54" t="s">
+      <c r="G26" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H26" s="54" t="s">
+      <c r="H26" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I26" s="54" t="s">
+      <c r="I26" s="45" t="s">
         <v>214</v>
       </c>
-      <c r="J26" s="54">
+      <c r="J26" s="45">
         <v>9</v>
       </c>
-      <c r="K26" s="54">
+      <c r="K26" s="45">
         <v>1</v>
       </c>
-      <c r="L26" s="54" t="s">
+      <c r="L26" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M26" s="54">
+      <c r="M26" s="45">
         <v>51</v>
       </c>
-      <c r="N26" s="54">
+      <c r="N26" s="45">
         <v>622</v>
       </c>
-      <c r="O26" s="54">
+      <c r="O26" s="45">
         <v>838</v>
       </c>
-      <c r="P26" s="54" t="s">
+      <c r="P26" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q26" s="54">
+      <c r="Q26" s="45">
         <v>9</v>
       </c>
-      <c r="R26" s="41"/>
+      <c r="R26" s="3"/>
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
-      <c r="V26" s="30"/>
-    </row>
-    <row r="27" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A27" s="54" t="s">
+    </row>
+    <row r="27" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A27" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="54">
+      <c r="B27" s="45">
         <v>2018</v>
       </c>
-      <c r="C27" s="54" t="s">
+      <c r="C27" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="54" t="s">
+      <c r="D27" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="54" t="s">
+      <c r="E27" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F27" s="54" t="s">
+      <c r="F27" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G27" s="54" t="s">
+      <c r="G27" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H27" s="54" t="s">
+      <c r="H27" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I27" s="54" t="s">
+      <c r="I27" s="45" t="s">
         <v>215</v>
       </c>
-      <c r="J27" s="54">
+      <c r="J27" s="45">
         <v>9</v>
       </c>
-      <c r="K27" s="54">
+      <c r="K27" s="45">
         <v>1</v>
       </c>
-      <c r="L27" s="54" t="s">
+      <c r="L27" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M27" s="54">
+      <c r="M27" s="45">
         <v>14</v>
       </c>
-      <c r="N27" s="54">
+      <c r="N27" s="45">
         <v>95</v>
       </c>
-      <c r="O27" s="54">
+      <c r="O27" s="45">
         <v>838</v>
       </c>
-      <c r="P27" s="54" t="s">
+      <c r="P27" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q27" s="54">
+      <c r="Q27" s="45">
         <v>9</v>
       </c>
-      <c r="R27" s="41"/>
+      <c r="R27" s="3"/>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
-      <c r="V27" s="30"/>
-    </row>
-    <row r="28" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A28" s="54" t="s">
+    </row>
+    <row r="28" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A28" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="54">
+      <c r="B28" s="45">
         <v>2018</v>
       </c>
-      <c r="C28" s="54" t="s">
+      <c r="C28" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D28" s="54" t="s">
+      <c r="D28" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E28" s="54" t="s">
+      <c r="E28" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F28" s="54" t="s">
+      <c r="F28" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G28" s="54" t="s">
+      <c r="G28" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H28" s="54" t="s">
+      <c r="H28" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I28" s="54" t="s">
+      <c r="I28" s="45" t="s">
         <v>216</v>
       </c>
-      <c r="J28" s="54">
+      <c r="J28" s="45">
         <v>9</v>
       </c>
-      <c r="K28" s="54">
+      <c r="K28" s="45">
         <v>1</v>
       </c>
-      <c r="L28" s="54" t="s">
+      <c r="L28" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M28" s="54">
+      <c r="M28" s="45">
         <v>69</v>
       </c>
-      <c r="N28" s="54">
+      <c r="N28" s="45">
         <v>742</v>
       </c>
-      <c r="O28" s="54">
+      <c r="O28" s="45">
         <v>838</v>
       </c>
-      <c r="P28" s="54" t="s">
+      <c r="P28" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q28" s="54">
+      <c r="Q28" s="45">
         <v>9</v>
       </c>
-      <c r="R28" s="41"/>
+      <c r="R28" s="3"/>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
-      <c r="V28" s="30"/>
-    </row>
-    <row r="29" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A29" s="54" t="s">
+    </row>
+    <row r="29" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A29" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="54">
+      <c r="B29" s="45">
         <v>2018</v>
       </c>
-      <c r="C29" s="54" t="s">
+      <c r="C29" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="54" t="s">
+      <c r="D29" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E29" s="54" t="s">
+      <c r="E29" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F29" s="54" t="s">
+      <c r="F29" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G29" s="54" t="s">
+      <c r="G29" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H29" s="54" t="s">
+      <c r="H29" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I29" s="54" t="s">
+      <c r="I29" s="45" t="s">
         <v>217</v>
       </c>
-      <c r="J29" s="54">
+      <c r="J29" s="45">
         <v>9</v>
       </c>
-      <c r="K29" s="54">
+      <c r="K29" s="45">
         <v>1</v>
       </c>
-      <c r="L29" s="54" t="s">
+      <c r="L29" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M29" s="54">
+      <c r="M29" s="45">
         <v>62</v>
       </c>
-      <c r="N29" s="54">
+      <c r="N29" s="45">
         <v>529</v>
       </c>
-      <c r="O29" s="54">
+      <c r="O29" s="45">
         <v>838</v>
       </c>
-      <c r="P29" s="54" t="s">
+      <c r="P29" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q29" s="54">
+      <c r="Q29" s="45">
         <v>9</v>
       </c>
-      <c r="R29" s="41"/>
+      <c r="R29" s="3"/>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
-      <c r="V29" s="30"/>
-    </row>
-    <row r="30" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A30" s="54" t="s">
+    </row>
+    <row r="30" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A30" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="54">
+      <c r="B30" s="45">
         <v>2018</v>
       </c>
-      <c r="C30" s="54" t="s">
+      <c r="C30" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D30" s="54" t="s">
+      <c r="D30" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E30" s="54" t="s">
+      <c r="E30" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F30" s="54" t="s">
+      <c r="F30" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G30" s="54" t="s">
+      <c r="G30" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H30" s="54" t="s">
+      <c r="H30" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I30" s="54" t="s">
+      <c r="I30" s="45" t="s">
         <v>218</v>
       </c>
-      <c r="J30" s="54">
+      <c r="J30" s="45">
         <v>9</v>
       </c>
-      <c r="K30" s="54">
+      <c r="K30" s="45">
         <v>1</v>
       </c>
-      <c r="L30" s="54" t="s">
+      <c r="L30" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M30" s="54">
+      <c r="M30" s="45">
         <v>21</v>
       </c>
-      <c r="N30" s="54">
+      <c r="N30" s="45">
         <v>302</v>
       </c>
-      <c r="O30" s="54">
+      <c r="O30" s="45">
         <v>838</v>
       </c>
-      <c r="P30" s="54" t="s">
+      <c r="P30" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q30" s="54">
+      <c r="Q30" s="45">
         <v>9</v>
       </c>
-      <c r="R30" s="41"/>
+      <c r="R30" s="3"/>
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
-      <c r="V30" s="30"/>
-    </row>
-    <row r="31" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A31" s="54" t="s">
+    </row>
+    <row r="31" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A31" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B31" s="54">
+      <c r="B31" s="45">
         <v>2018</v>
       </c>
-      <c r="C31" s="54" t="s">
+      <c r="C31" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="54" t="s">
+      <c r="D31" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E31" s="54" t="s">
+      <c r="E31" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F31" s="54" t="s">
+      <c r="F31" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G31" s="54" t="s">
+      <c r="G31" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H31" s="54" t="s">
+      <c r="H31" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I31" s="54" t="s">
+      <c r="I31" s="45" t="s">
         <v>219</v>
       </c>
-      <c r="J31" s="54">
+      <c r="J31" s="45">
         <v>9</v>
       </c>
-      <c r="K31" s="54">
+      <c r="K31" s="45">
         <v>1</v>
       </c>
-      <c r="L31" s="54" t="s">
+      <c r="L31" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M31" s="54">
+      <c r="M31" s="45">
         <v>31</v>
       </c>
-      <c r="N31" s="54">
+      <c r="N31" s="45">
         <v>215</v>
       </c>
-      <c r="O31" s="54">
+      <c r="O31" s="45">
         <v>838</v>
       </c>
-      <c r="P31" s="54" t="s">
+      <c r="P31" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q31" s="54">
+      <c r="Q31" s="45">
         <v>9</v>
       </c>
-      <c r="R31" s="41"/>
+      <c r="R31" s="3"/>
       <c r="S31" s="3"/>
       <c r="T31" s="3"/>
       <c r="U31" s="3"/>
-      <c r="V31" s="30"/>
-    </row>
-    <row r="32" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A32" s="54" t="s">
+    </row>
+    <row r="32" spans="1:21" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A32" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="54">
+      <c r="B32" s="45">
         <v>2018</v>
       </c>
-      <c r="C32" s="54" t="s">
+      <c r="C32" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="54" t="s">
+      <c r="D32" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E32" s="54" t="s">
+      <c r="E32" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F32" s="54" t="s">
+      <c r="F32" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G32" s="54" t="s">
+      <c r="G32" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H32" s="54" t="s">
+      <c r="H32" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I32" s="54" t="s">
+      <c r="I32" s="45" t="s">
         <v>220</v>
       </c>
-      <c r="J32" s="54">
+      <c r="J32" s="45">
         <v>9</v>
       </c>
-      <c r="K32" s="54">
+      <c r="K32" s="45">
         <v>1</v>
       </c>
-      <c r="L32" s="54" t="s">
+      <c r="L32" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M32" s="54">
+      <c r="M32" s="45">
         <v>50</v>
       </c>
-      <c r="N32" s="54">
+      <c r="N32" s="45">
         <v>621</v>
       </c>
-      <c r="O32" s="54">
+      <c r="O32" s="45">
         <v>838</v>
       </c>
-      <c r="P32" s="54" t="s">
+      <c r="P32" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q32" s="54">
+      <c r="Q32" s="45">
         <v>9</v>
       </c>
-      <c r="R32" s="41"/>
+      <c r="R32" s="3"/>
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
-      <c r="V32" s="30"/>
-    </row>
-    <row r="33" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A33" s="54" t="s">
+    </row>
+    <row r="33" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A33" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B33" s="54">
+      <c r="B33" s="45">
         <v>2018</v>
       </c>
-      <c r="C33" s="54" t="s">
+      <c r="C33" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="54" t="s">
+      <c r="D33" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E33" s="54" t="s">
+      <c r="E33" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F33" s="54" t="s">
+      <c r="F33" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G33" s="54" t="s">
+      <c r="G33" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H33" s="54" t="s">
+      <c r="H33" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I33" s="54" t="s">
+      <c r="I33" s="45" t="s">
         <v>221</v>
       </c>
-      <c r="J33" s="54">
+      <c r="J33" s="45">
         <v>9</v>
       </c>
-      <c r="K33" s="54">
+      <c r="K33" s="45">
         <v>1</v>
       </c>
-      <c r="L33" s="54" t="s">
+      <c r="L33" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M33" s="54">
+      <c r="M33" s="45">
         <v>26</v>
       </c>
-      <c r="N33" s="54">
+      <c r="N33" s="45">
         <v>188</v>
       </c>
-      <c r="O33" s="54">
+      <c r="O33" s="45">
         <v>838</v>
       </c>
-      <c r="P33" s="54" t="s">
+      <c r="P33" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q33" s="54">
+      <c r="Q33" s="45">
         <v>9</v>
       </c>
-      <c r="R33" s="41"/>
+      <c r="R33" s="3"/>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
-      <c r="V33" s="30"/>
-    </row>
-    <row r="34" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A34" s="54" t="s">
+    </row>
+    <row r="34" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A34" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B34" s="54">
+      <c r="B34" s="45">
         <v>2018</v>
       </c>
-      <c r="C34" s="54" t="s">
+      <c r="C34" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="54" t="s">
+      <c r="D34" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E34" s="54" t="s">
+      <c r="E34" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F34" s="54" t="s">
+      <c r="F34" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G34" s="54" t="s">
+      <c r="G34" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H34" s="54" t="s">
+      <c r="H34" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I34" s="54" t="s">
+      <c r="I34" s="45" t="s">
         <v>222</v>
       </c>
-      <c r="J34" s="54">
+      <c r="J34" s="45">
         <v>9</v>
       </c>
-      <c r="K34" s="54">
+      <c r="K34" s="45">
         <v>1</v>
       </c>
-      <c r="L34" s="54" t="s">
+      <c r="L34" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M34" s="54">
+      <c r="M34" s="45">
         <v>5</v>
       </c>
-      <c r="N34" s="54">
+      <c r="N34" s="45">
         <v>27</v>
       </c>
-      <c r="O34" s="54">
+      <c r="O34" s="45">
         <v>838</v>
       </c>
-      <c r="P34" s="54" t="s">
+      <c r="P34" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q34" s="54">
+      <c r="Q34" s="45">
         <v>9</v>
       </c>
-      <c r="R34" s="41"/>
+      <c r="R34" s="3"/>
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
-      <c r="V34" s="30"/>
-    </row>
-    <row r="35" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A35" s="54" t="s">
+    </row>
+    <row r="35" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A35" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B35" s="54">
+      <c r="B35" s="45">
         <v>2018</v>
       </c>
-      <c r="C35" s="54" t="s">
+      <c r="C35" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D35" s="54" t="s">
+      <c r="D35" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E35" s="54" t="s">
+      <c r="E35" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F35" s="54" t="s">
+      <c r="F35" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G35" s="54" t="s">
+      <c r="G35" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H35" s="54" t="s">
+      <c r="H35" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I35" s="54" t="s">
+      <c r="I35" s="45" t="s">
         <v>223</v>
       </c>
-      <c r="J35" s="54">
+      <c r="J35" s="45">
         <v>9</v>
       </c>
-      <c r="K35" s="54">
+      <c r="K35" s="45">
         <v>1</v>
       </c>
-      <c r="L35" s="54" t="s">
+      <c r="L35" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M35" s="54">
+      <c r="M35" s="45">
         <v>27</v>
       </c>
-      <c r="N35" s="54">
+      <c r="N35" s="45">
         <v>175</v>
       </c>
-      <c r="O35" s="54">
+      <c r="O35" s="45">
         <v>838</v>
       </c>
-      <c r="P35" s="54" t="s">
+      <c r="P35" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q35" s="54">
+      <c r="Q35" s="45">
         <v>9</v>
       </c>
-      <c r="R35" s="41"/>
+      <c r="R35" s="3"/>
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
       <c r="U35" s="3"/>
-      <c r="V35" s="30"/>
-    </row>
-    <row r="36" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A36" s="54" t="s">
+    </row>
+    <row r="36" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A36" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B36" s="54">
+      <c r="B36" s="45">
         <v>2018</v>
       </c>
-      <c r="C36" s="54" t="s">
+      <c r="C36" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D36" s="54" t="s">
+      <c r="D36" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E36" s="54" t="s">
+      <c r="E36" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F36" s="54" t="s">
+      <c r="F36" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G36" s="54" t="s">
+      <c r="G36" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H36" s="54" t="s">
+      <c r="H36" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I36" s="54" t="s">
+      <c r="I36" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="J36" s="54">
+      <c r="J36" s="45">
         <v>9</v>
       </c>
-      <c r="K36" s="54">
+      <c r="K36" s="45">
         <v>1</v>
       </c>
-      <c r="L36" s="54" t="s">
+      <c r="L36" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M36" s="54">
+      <c r="M36" s="45">
         <v>4</v>
       </c>
-      <c r="N36" s="54">
+      <c r="N36" s="45">
         <v>40</v>
       </c>
-      <c r="O36" s="54">
+      <c r="O36" s="45">
         <v>838</v>
       </c>
-      <c r="P36" s="54" t="s">
+      <c r="P36" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q36" s="54">
+      <c r="Q36" s="45">
         <v>9</v>
       </c>
-      <c r="R36" s="41"/>
+      <c r="R36" s="3"/>
       <c r="S36" s="3"/>
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
-      <c r="V36" s="30"/>
-    </row>
-    <row r="37" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A37" s="54" t="s">
+    </row>
+    <row r="37" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A37" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B37" s="54">
+      <c r="B37" s="45">
         <v>2018</v>
       </c>
-      <c r="C37" s="54" t="s">
+      <c r="C37" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D37" s="54" t="s">
+      <c r="D37" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E37" s="54" t="s">
+      <c r="E37" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F37" s="54" t="s">
+      <c r="F37" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G37" s="54" t="s">
+      <c r="G37" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H37" s="54" t="s">
+      <c r="H37" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I37" s="54" t="s">
+      <c r="I37" s="45" t="s">
         <v>225</v>
       </c>
-      <c r="J37" s="54">
+      <c r="J37" s="45">
         <v>9</v>
       </c>
-      <c r="K37" s="54">
+      <c r="K37" s="45">
         <v>1</v>
       </c>
-      <c r="L37" s="54" t="s">
+      <c r="L37" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M37" s="54">
+      <c r="M37" s="45">
         <v>33</v>
       </c>
-      <c r="N37" s="54">
+      <c r="N37" s="45">
         <v>188</v>
       </c>
-      <c r="O37" s="54">
+      <c r="O37" s="45">
         <v>838</v>
       </c>
-      <c r="P37" s="54" t="s">
+      <c r="P37" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q37" s="54">
+      <c r="Q37" s="45">
         <v>9</v>
       </c>
-      <c r="R37" s="41"/>
+      <c r="R37" s="3"/>
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
-      <c r="V37" s="30"/>
-    </row>
-    <row r="38" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A38" s="54" t="s">
+    </row>
+    <row r="38" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A38" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="54">
+      <c r="B38" s="45">
         <v>2018</v>
       </c>
-      <c r="C38" s="54" t="s">
+      <c r="C38" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="54" t="s">
+      <c r="D38" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E38" s="54" t="s">
+      <c r="E38" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F38" s="54" t="s">
+      <c r="F38" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G38" s="54" t="s">
+      <c r="G38" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H38" s="54" t="s">
+      <c r="H38" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I38" s="54" t="s">
+      <c r="I38" s="45" t="s">
         <v>226</v>
       </c>
-      <c r="J38" s="54">
+      <c r="J38" s="45">
         <v>9</v>
       </c>
-      <c r="K38" s="54">
+      <c r="K38" s="45">
         <v>1</v>
       </c>
-      <c r="L38" s="54" t="s">
+      <c r="L38" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M38" s="54">
+      <c r="M38" s="45">
         <v>50</v>
       </c>
-      <c r="N38" s="54">
+      <c r="N38" s="45">
         <v>645</v>
       </c>
-      <c r="O38" s="54">
+      <c r="O38" s="45">
         <v>838</v>
       </c>
-      <c r="P38" s="54" t="s">
+      <c r="P38" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q38" s="54">
+      <c r="Q38" s="45">
         <v>9</v>
       </c>
-      <c r="R38" s="41"/>
+      <c r="R38" s="3"/>
       <c r="S38" s="3"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
-      <c r="V38" s="30"/>
-    </row>
-    <row r="39" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A39" s="54" t="s">
+    </row>
+    <row r="39" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A39" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B39" s="54">
+      <c r="B39" s="45">
         <v>2018</v>
       </c>
-      <c r="C39" s="54" t="s">
+      <c r="C39" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D39" s="54" t="s">
+      <c r="D39" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E39" s="54" t="s">
+      <c r="E39" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F39" s="54" t="s">
+      <c r="F39" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G39" s="54" t="s">
+      <c r="G39" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H39" s="54" t="s">
+      <c r="H39" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I39" s="54" t="s">
+      <c r="I39" s="45" t="s">
         <v>227</v>
       </c>
-      <c r="J39" s="54">
+      <c r="J39" s="45">
         <v>9</v>
       </c>
-      <c r="K39" s="54">
+      <c r="K39" s="45">
         <v>1</v>
       </c>
-      <c r="L39" s="54" t="s">
+      <c r="L39" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M39" s="54">
+      <c r="M39" s="45">
         <v>24</v>
       </c>
-      <c r="N39" s="54">
+      <c r="N39" s="45">
         <v>115</v>
       </c>
-      <c r="O39" s="54">
+      <c r="O39" s="45">
         <v>838</v>
       </c>
-      <c r="P39" s="54" t="s">
+      <c r="P39" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q39" s="54">
+      <c r="Q39" s="45">
         <v>9</v>
       </c>
-      <c r="R39" s="41"/>
+      <c r="R39" s="3"/>
       <c r="S39" s="3"/>
       <c r="T39" s="3"/>
       <c r="U39" s="3"/>
-      <c r="V39" s="30"/>
-    </row>
-    <row r="40" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A40" s="54" t="s">
+    </row>
+    <row r="40" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A40" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="54">
+      <c r="B40" s="45">
         <v>2018</v>
       </c>
-      <c r="C40" s="54" t="s">
+      <c r="C40" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D40" s="54" t="s">
+      <c r="D40" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E40" s="54" t="s">
+      <c r="E40" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F40" s="54" t="s">
+      <c r="F40" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G40" s="54" t="s">
+      <c r="G40" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H40" s="54" t="s">
+      <c r="H40" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I40" s="54" t="s">
+      <c r="I40" s="45" t="s">
         <v>228</v>
       </c>
-      <c r="J40" s="54">
+      <c r="J40" s="45">
         <v>9</v>
       </c>
-      <c r="K40" s="54">
+      <c r="K40" s="45">
         <v>1</v>
       </c>
-      <c r="L40" s="54" t="s">
+      <c r="L40" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M40" s="54">
+      <c r="M40" s="45">
         <v>59</v>
       </c>
-      <c r="N40" s="54">
+      <c r="N40" s="45">
         <v>715</v>
       </c>
-      <c r="O40" s="54">
+      <c r="O40" s="45">
         <v>838</v>
       </c>
-      <c r="P40" s="54" t="s">
+      <c r="P40" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q40" s="54">
+      <c r="Q40" s="45">
         <v>9</v>
       </c>
-      <c r="R40" s="41"/>
+      <c r="R40" s="3"/>
       <c r="S40" s="3"/>
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
-      <c r="V40" s="30"/>
-    </row>
-    <row r="41" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A41" s="54" t="s">
+    </row>
+    <row r="41" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A41" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B41" s="54">
+      <c r="B41" s="45">
         <v>2018</v>
       </c>
-      <c r="C41" s="54" t="s">
+      <c r="C41" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D41" s="54" t="s">
+      <c r="D41" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E41" s="54" t="s">
+      <c r="E41" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F41" s="54" t="s">
+      <c r="F41" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G41" s="54" t="s">
+      <c r="G41" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H41" s="54" t="s">
+      <c r="H41" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I41" s="54" t="s">
+      <c r="I41" s="45" t="s">
         <v>229</v>
       </c>
-      <c r="J41" s="54">
+      <c r="J41" s="45">
         <v>9</v>
       </c>
-      <c r="K41" s="54">
+      <c r="K41" s="45">
         <v>1</v>
       </c>
-      <c r="L41" s="54" t="s">
+      <c r="L41" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M41" s="54">
+      <c r="M41" s="45">
         <v>7</v>
       </c>
-      <c r="N41" s="54">
+      <c r="N41" s="45">
         <v>25</v>
       </c>
-      <c r="O41" s="54">
+      <c r="O41" s="45">
         <v>838</v>
       </c>
-      <c r="P41" s="54" t="s">
+      <c r="P41" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q41" s="54">
+      <c r="Q41" s="45">
         <v>9</v>
       </c>
-      <c r="R41" s="41"/>
+      <c r="R41" s="3"/>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
-      <c r="V41" s="30"/>
-    </row>
-    <row r="42" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A42" s="54" t="s">
+    </row>
+    <row r="42" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A42" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B42" s="54">
+      <c r="B42" s="45">
         <v>2018</v>
       </c>
-      <c r="C42" s="54" t="s">
+      <c r="C42" s="45" t="s">
         <v>55</v>
       </c>
-      <c r="D42" s="54" t="s">
+      <c r="D42" s="45" t="s">
         <v>56</v>
       </c>
-      <c r="E42" s="54" t="s">
+      <c r="E42" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="F42" s="54" t="s">
+      <c r="F42" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="G42" s="54" t="s">
+      <c r="G42" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="H42" s="54" t="s">
+      <c r="H42" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="I42" s="54" t="s">
+      <c r="I42" s="45" t="s">
         <v>230</v>
       </c>
-      <c r="J42" s="54">
+      <c r="J42" s="45">
         <v>9</v>
       </c>
-      <c r="K42" s="54">
+      <c r="K42" s="45">
         <v>1</v>
       </c>
-      <c r="L42" s="54" t="s">
+      <c r="L42" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="M42" s="54">
+      <c r="M42" s="45">
         <v>76</v>
       </c>
-      <c r="N42" s="54">
+      <c r="N42" s="45">
         <v>798</v>
       </c>
-      <c r="O42" s="54">
+      <c r="O42" s="45">
         <v>838</v>
       </c>
-      <c r="P42" s="54" t="s">
+      <c r="P42" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="Q42" s="54">
+      <c r="Q42" s="45">
         <v>9</v>
       </c>
-      <c r="R42" s="41"/>
+      <c r="R42" s="3"/>
       <c r="S42" s="3"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
-      <c r="V42" s="30"/>
-    </row>
-    <row r="43" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A43" s="51" t="s">
+    </row>
+    <row r="43" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A43" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B43" s="51">
+      <c r="B43" s="42">
         <v>2018</v>
       </c>
-      <c r="C43" s="51" t="s">
+      <c r="C43" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="D43" s="51" t="s">
+      <c r="D43" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="E43" s="51" t="s">
+      <c r="E43" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="F43" s="52" t="s">
+      <c r="F43" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="G43" s="51" t="s">
+      <c r="G43" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="H43" s="51" t="s">
+      <c r="H43" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="I43" s="51" t="s">
+      <c r="I43" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="J43" s="52">
+      <c r="J43" s="43">
         <v>9</v>
       </c>
-      <c r="K43" s="51">
+      <c r="K43" s="42">
         <v>1</v>
       </c>
-      <c r="L43" s="51" t="s">
+      <c r="L43" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="M43" s="51">
+      <c r="M43" s="42">
         <v>33</v>
       </c>
-      <c r="N43" s="51">
+      <c r="N43" s="42">
         <v>548</v>
       </c>
-      <c r="O43" s="51">
+      <c r="O43" s="42">
         <v>838</v>
       </c>
-      <c r="P43" s="51" t="s">
+      <c r="P43" s="42" t="s">
         <v>62</v>
       </c>
       <c r="Q43" s="3">
         <v>150</v>
       </c>
-      <c r="R43" s="41">
+      <c r="R43" s="3">
         <v>9</v>
       </c>
-      <c r="S43" s="51" t="s">
+      <c r="S43" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="T43" s="51" t="b">
+      <c r="T43" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="U43" s="51" t="b">
+      <c r="U43" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="V43" s="51" t="s">
+      <c r="V43" s="42" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="44" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A44" s="51" t="s">
+    <row r="44" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A44" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B44" s="51">
+      <c r="B44" s="42">
         <v>2018</v>
       </c>
-      <c r="C44" s="51" t="s">
+      <c r="C44" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="D44" s="51" t="s">
+      <c r="D44" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="E44" s="51" t="s">
+      <c r="E44" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="F44" s="52" t="s">
+      <c r="F44" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="G44" s="51" t="s">
+      <c r="G44" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="H44" s="51" t="s">
+      <c r="H44" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="I44" s="51" t="s">
+      <c r="I44" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="J44" s="52">
+      <c r="J44" s="43">
         <v>9</v>
       </c>
-      <c r="K44" s="51">
+      <c r="K44" s="42">
         <v>1</v>
       </c>
-      <c r="L44" s="51" t="s">
+      <c r="L44" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="M44" s="51">
+      <c r="M44" s="42">
         <v>13</v>
       </c>
-      <c r="N44" s="51">
+      <c r="N44" s="42">
         <v>133</v>
       </c>
-      <c r="O44" s="51">
+      <c r="O44" s="42">
         <v>838</v>
       </c>
-      <c r="P44" s="51" t="s">
+      <c r="P44" s="42" t="s">
         <v>62</v>
       </c>
       <c r="Q44" s="3">
         <v>150</v>
       </c>
-      <c r="R44" s="41">
+      <c r="R44" s="3">
         <v>9</v>
       </c>
-      <c r="S44" s="51" t="s">
+      <c r="S44" s="42" t="s">
         <v>145</v>
       </c>
-      <c r="T44" s="51" t="b">
+      <c r="T44" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="U44" s="51" t="b">
+      <c r="U44" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="V44" s="51" t="s">
+      <c r="V44" s="42" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="45" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A45" s="51" t="s">
+    <row r="45" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A45" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B45" s="51">
+      <c r="B45" s="42">
         <v>2018</v>
       </c>
-      <c r="C45" s="51" t="s">
+      <c r="C45" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="D45" s="51" t="s">
+      <c r="D45" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="E45" s="51" t="s">
+      <c r="E45" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="F45" s="52" t="s">
+      <c r="F45" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="G45" s="51" t="s">
+      <c r="G45" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="H45" s="51" t="s">
+      <c r="H45" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="I45" s="51" t="s">
+      <c r="I45" s="42" t="s">
         <v>66</v>
       </c>
-      <c r="J45" s="52">
+      <c r="J45" s="43">
         <v>9</v>
       </c>
-      <c r="K45" s="51">
+      <c r="K45" s="42">
         <v>1</v>
       </c>
-      <c r="L45" s="51" t="s">
+      <c r="L45" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="M45" s="51">
+      <c r="M45" s="42">
         <v>13</v>
       </c>
-      <c r="N45" s="51">
+      <c r="N45" s="42">
         <v>44</v>
       </c>
-      <c r="O45" s="51">
+      <c r="O45" s="42">
         <v>838</v>
       </c>
-      <c r="P45" s="51" t="s">
+      <c r="P45" s="42" t="s">
         <v>62</v>
       </c>
       <c r="Q45" s="3">
         <v>150</v>
       </c>
-      <c r="R45" s="41">
+      <c r="R45" s="3">
         <v>9</v>
       </c>
-      <c r="S45" s="51" t="s">
+      <c r="S45" s="42" t="s">
         <v>146</v>
       </c>
-      <c r="T45" s="51" t="b">
+      <c r="T45" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="U45" s="51" t="b">
+      <c r="U45" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="V45" s="51" t="s">
+      <c r="V45" s="42" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="46" spans="1:22" s="50" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A46" s="51" t="s">
+    <row r="46" spans="1:22" s="30" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A46" s="42" t="s">
         <v>54</v>
       </c>
-      <c r="B46" s="51">
+      <c r="B46" s="42">
         <v>2018</v>
       </c>
-      <c r="C46" s="51" t="s">
+      <c r="C46" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="D46" s="51" t="s">
+      <c r="D46" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="E46" s="51" t="s">
+      <c r="E46" s="42" t="s">
         <v>57</v>
       </c>
-      <c r="F46" s="52" t="s">
+      <c r="F46" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="G46" s="51" t="s">
+      <c r="G46" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="H46" s="51" t="s">
+      <c r="H46" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="I46" s="51" t="s">
+      <c r="I46" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="J46" s="52">
+      <c r="J46" s="43">
         <v>9</v>
       </c>
-      <c r="K46" s="51">
+      <c r="K46" s="42">
         <v>1</v>
       </c>
-      <c r="L46" s="51" t="s">
+      <c r="L46" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="M46" s="51">
+      <c r="M46" s="42">
         <v>24</v>
       </c>
-      <c r="N46" s="51">
+      <c r="N46" s="42">
         <v>112</v>
       </c>
-      <c r="O46" s="51">
+      <c r="O46" s="42">
         <v>838</v>
       </c>
-      <c r="P46" s="51" t="s">
+      <c r="P46" s="42" t="s">
         <v>62</v>
       </c>
       <c r="Q46" s="3">
         <v>150</v>
       </c>
-      <c r="R46" s="41">
+      <c r="R46" s="3">
         <v>9</v>
       </c>
-      <c r="S46" s="51" t="s">
+      <c r="S46" s="42" t="s">
         <v>147</v>
       </c>
-      <c r="T46" s="51" t="b">
+      <c r="T46" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="U46" s="51" t="b">
+      <c r="U46" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="V46" s="51" t="s">
+      <c r="V46" s="42" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="47" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A47" s="35" t="s">
+      <c r="A47" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="35">
+      <c r="B47" s="32">
         <v>2003</v>
       </c>
-      <c r="C47" s="35" t="s">
+      <c r="C47" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D47" s="35" t="s">
+      <c r="D47" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E47" s="35" t="s">
+      <c r="E47" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F47" s="36" t="s">
+      <c r="F47" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G47" s="35" t="s">
+      <c r="G47" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H47" s="35" t="s">
+      <c r="H47" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I47" s="35" t="s">
+      <c r="I47" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="J47" s="36">
+      <c r="J47" s="33">
         <v>9</v>
       </c>
-      <c r="K47" s="35">
+      <c r="K47" s="32">
         <v>2</v>
       </c>
-      <c r="L47" s="35">
+      <c r="L47" s="32">
         <v>9</v>
       </c>
-      <c r="M47" s="35">
+      <c r="M47" s="32">
         <v>24</v>
       </c>
-      <c r="N47" s="35">
+      <c r="N47" s="32">
         <v>89</v>
       </c>
-      <c r="O47" s="35">
+      <c r="O47" s="32">
         <v>89</v>
       </c>
-      <c r="P47" s="35" t="s">
+      <c r="P47" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q47" s="35">
+      <c r="Q47" s="32">
         <v>27</v>
       </c>
-      <c r="R47" s="46">
+      <c r="R47" s="4">
         <v>9</v>
       </c>
-      <c r="S47" s="35" t="s">
+      <c r="S47" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="T47" s="35" t="b">
+      <c r="T47" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U47" s="35" t="b">
+      <c r="U47" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V47" s="40" t="s">
+      <c r="V47" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="48" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A48" s="35" t="s">
+      <c r="A48" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B48" s="35">
+      <c r="B48" s="32">
         <v>2003</v>
       </c>
-      <c r="C48" s="35" t="s">
+      <c r="C48" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D48" s="35" t="s">
+      <c r="D48" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E48" s="35" t="s">
+      <c r="E48" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F48" s="36" t="s">
+      <c r="F48" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G48" s="35" t="s">
+      <c r="G48" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H48" s="35" t="s">
+      <c r="H48" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I48" s="35" t="s">
+      <c r="I48" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="J48" s="36">
+      <c r="J48" s="33">
         <v>9</v>
       </c>
-      <c r="K48" s="35">
+      <c r="K48" s="32">
         <v>2</v>
       </c>
-      <c r="L48" s="35">
+      <c r="L48" s="32">
         <v>9</v>
       </c>
-      <c r="M48" s="35">
+      <c r="M48" s="32">
         <v>19</v>
       </c>
-      <c r="N48" s="35">
+      <c r="N48" s="32">
         <v>70</v>
       </c>
-      <c r="O48" s="35">
+      <c r="O48" s="32">
         <v>89</v>
       </c>
-      <c r="P48" s="35" t="s">
+      <c r="P48" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q48" s="35">
+      <c r="Q48" s="32">
         <v>27</v>
       </c>
-      <c r="R48" s="46">
+      <c r="R48" s="4">
         <v>9</v>
       </c>
-      <c r="S48" s="35" t="s">
+      <c r="S48" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="T48" s="35" t="b">
+      <c r="T48" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U48" s="35" t="b">
+      <c r="U48" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V48" s="40" t="s">
+      <c r="V48" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="49" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A49" s="35" t="s">
+      <c r="A49" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B49" s="35">
+      <c r="B49" s="32">
         <v>2003</v>
       </c>
-      <c r="C49" s="35" t="s">
+      <c r="C49" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D49" s="35" t="s">
+      <c r="D49" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E49" s="35" t="s">
+      <c r="E49" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F49" s="36" t="s">
+      <c r="F49" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G49" s="35" t="s">
+      <c r="G49" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H49" s="35" t="s">
+      <c r="H49" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I49" s="35" t="s">
+      <c r="I49" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="J49" s="36">
+      <c r="J49" s="33">
         <v>9</v>
       </c>
-      <c r="K49" s="35">
+      <c r="K49" s="32">
         <v>2</v>
       </c>
-      <c r="L49" s="35">
+      <c r="L49" s="32">
         <v>9</v>
       </c>
-      <c r="M49" s="35">
+      <c r="M49" s="32">
         <v>1</v>
       </c>
-      <c r="N49" s="35">
+      <c r="N49" s="32">
         <v>13</v>
       </c>
-      <c r="O49" s="35">
+      <c r="O49" s="32">
         <v>89</v>
       </c>
-      <c r="P49" s="35" t="s">
+      <c r="P49" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q49" s="35">
+      <c r="Q49" s="32">
         <v>27</v>
       </c>
-      <c r="R49" s="46">
+      <c r="R49" s="4">
         <v>9</v>
       </c>
-      <c r="S49" s="35" t="s">
+      <c r="S49" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="T49" s="35" t="b">
+      <c r="T49" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U49" s="35" t="b">
+      <c r="U49" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V49" s="40" t="s">
+      <c r="V49" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="50" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A50" s="35" t="s">
+      <c r="A50" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B50" s="35">
+      <c r="B50" s="32">
         <v>2003</v>
       </c>
-      <c r="C50" s="35" t="s">
+      <c r="C50" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D50" s="35" t="s">
+      <c r="D50" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E50" s="35" t="s">
+      <c r="E50" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F50" s="36" t="s">
+      <c r="F50" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G50" s="35" t="s">
+      <c r="G50" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H50" s="35" t="s">
+      <c r="H50" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I50" s="35" t="s">
+      <c r="I50" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="J50" s="36">
+      <c r="J50" s="33">
         <v>9</v>
       </c>
-      <c r="K50" s="35">
+      <c r="K50" s="32">
         <v>2</v>
       </c>
-      <c r="L50" s="35">
+      <c r="L50" s="32">
         <v>9</v>
       </c>
-      <c r="M50" s="35">
+      <c r="M50" s="32">
         <v>15</v>
       </c>
-      <c r="N50" s="35">
+      <c r="N50" s="32">
         <v>30</v>
       </c>
-      <c r="O50" s="35">
+      <c r="O50" s="32">
         <v>89</v>
       </c>
-      <c r="P50" s="35" t="s">
+      <c r="P50" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q50" s="35">
+      <c r="Q50" s="32">
         <v>27</v>
       </c>
-      <c r="R50" s="46">
+      <c r="R50" s="4">
         <v>9</v>
       </c>
-      <c r="S50" s="35" t="s">
+      <c r="S50" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="T50" s="35" t="b">
+      <c r="T50" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U50" s="35" t="b">
+      <c r="U50" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V50" s="40" t="s">
+      <c r="V50" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="51" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A51" s="35" t="s">
+      <c r="A51" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B51" s="35">
+      <c r="B51" s="32">
         <v>2003</v>
       </c>
-      <c r="C51" s="35" t="s">
+      <c r="C51" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D51" s="35" t="s">
+      <c r="D51" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E51" s="35" t="s">
+      <c r="E51" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F51" s="36" t="s">
+      <c r="F51" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G51" s="35" t="s">
+      <c r="G51" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H51" s="35" t="s">
+      <c r="H51" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I51" s="35" t="s">
+      <c r="I51" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="J51" s="36">
+      <c r="J51" s="33">
         <v>9</v>
       </c>
-      <c r="K51" s="35">
+      <c r="K51" s="32">
         <v>2</v>
       </c>
-      <c r="L51" s="35">
+      <c r="L51" s="32">
         <v>9</v>
       </c>
-      <c r="M51" s="35">
+      <c r="M51" s="32">
         <v>5</v>
       </c>
-      <c r="N51" s="35">
+      <c r="N51" s="32">
         <v>53</v>
       </c>
-      <c r="O51" s="35">
+      <c r="O51" s="32">
         <v>89</v>
       </c>
-      <c r="P51" s="35" t="s">
+      <c r="P51" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q51" s="35">
+      <c r="Q51" s="32">
         <v>27</v>
       </c>
-      <c r="R51" s="46">
+      <c r="R51" s="4">
         <v>9</v>
       </c>
-      <c r="S51" s="35" t="s">
+      <c r="S51" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="T51" s="35" t="b">
+      <c r="T51" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U51" s="35" t="b">
+      <c r="U51" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V51" s="40" t="s">
+      <c r="V51" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="52" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A52" s="35" t="s">
+      <c r="A52" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B52" s="35">
+      <c r="B52" s="32">
         <v>2003</v>
       </c>
-      <c r="C52" s="35" t="s">
+      <c r="C52" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D52" s="35" t="s">
+      <c r="D52" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E52" s="35" t="s">
+      <c r="E52" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F52" s="36" t="s">
+      <c r="F52" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G52" s="35" t="s">
+      <c r="G52" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H52" s="35" t="s">
+      <c r="H52" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I52" s="35" t="s">
+      <c r="I52" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="J52" s="36">
+      <c r="J52" s="33">
         <v>9</v>
       </c>
-      <c r="K52" s="35">
+      <c r="K52" s="32">
         <v>2</v>
       </c>
-      <c r="L52" s="35">
+      <c r="L52" s="32">
         <v>9</v>
       </c>
-      <c r="M52" s="35">
+      <c r="M52" s="32">
         <v>2</v>
       </c>
-      <c r="N52" s="35">
+      <c r="N52" s="32">
         <v>40</v>
       </c>
-      <c r="O52" s="35">
+      <c r="O52" s="32">
         <v>89</v>
       </c>
-      <c r="P52" s="35" t="s">
+      <c r="P52" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q52" s="35">
+      <c r="Q52" s="32">
         <v>27</v>
       </c>
-      <c r="R52" s="46">
+      <c r="R52" s="4">
         <v>9</v>
       </c>
-      <c r="S52" s="35" t="s">
+      <c r="S52" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="T52" s="35" t="b">
+      <c r="T52" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U52" s="35" t="b">
+      <c r="U52" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V52" s="40" t="s">
+      <c r="V52" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="53" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A53" s="35" t="s">
+      <c r="A53" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="B53" s="35">
+      <c r="B53" s="32">
         <v>2003</v>
       </c>
-      <c r="C53" s="35" t="s">
+      <c r="C53" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D53" s="35" t="s">
+      <c r="D53" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="E53" s="35" t="s">
+      <c r="E53" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="F53" s="36" t="s">
+      <c r="F53" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="G53" s="35" t="s">
+      <c r="G53" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="H53" s="35" t="s">
+      <c r="H53" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="I53" s="35" t="s">
+      <c r="I53" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="J53" s="36">
+      <c r="J53" s="33">
         <v>9</v>
       </c>
-      <c r="K53" s="35">
+      <c r="K53" s="32">
         <v>2</v>
       </c>
-      <c r="L53" s="35">
+      <c r="L53" s="32">
         <v>9</v>
       </c>
-      <c r="M53" s="35">
+      <c r="M53" s="32">
         <v>18</v>
       </c>
-      <c r="N53" s="35">
+      <c r="N53" s="32">
         <v>43</v>
       </c>
-      <c r="O53" s="35">
+      <c r="O53" s="32">
         <v>89</v>
       </c>
-      <c r="P53" s="35" t="s">
+      <c r="P53" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="Q53" s="35">
+      <c r="Q53" s="32">
         <v>27</v>
       </c>
-      <c r="R53" s="46">
+      <c r="R53" s="4">
         <v>9</v>
       </c>
-      <c r="S53" s="35" t="s">
+      <c r="S53" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="T53" s="35" t="b">
+      <c r="T53" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U53" s="35" t="b">
+      <c r="U53" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V53" s="40" t="s">
+      <c r="V53" s="37" t="s">
         <v>202</v>
       </c>
     </row>
@@ -18928,7 +18879,7 @@
       <c r="Q54" s="4">
         <v>71</v>
       </c>
-      <c r="R54" s="46">
+      <c r="R54" s="4">
         <v>9</v>
       </c>
       <c r="S54" s="4" t="s">
@@ -18993,7 +18944,7 @@
       <c r="Q55" s="4">
         <v>71</v>
       </c>
-      <c r="R55" s="46">
+      <c r="R55" s="4">
         <v>9</v>
       </c>
       <c r="S55" s="4" t="s">
@@ -19058,7 +19009,7 @@
       <c r="Q56" s="4">
         <v>71</v>
       </c>
-      <c r="R56" s="46">
+      <c r="R56" s="4">
         <v>9</v>
       </c>
       <c r="S56" s="4" t="s">
@@ -19123,7 +19074,7 @@
       <c r="Q57" s="4">
         <v>27</v>
       </c>
-      <c r="R57" s="46" t="s">
+      <c r="R57" s="4" t="s">
         <v>98</v>
       </c>
       <c r="S57" s="4" t="s">
@@ -19188,7 +19139,7 @@
       <c r="Q58" s="4">
         <v>27</v>
       </c>
-      <c r="R58" s="46" t="s">
+      <c r="R58" s="4" t="s">
         <v>98</v>
       </c>
       <c r="S58" s="4" t="s">
@@ -19256,7 +19207,7 @@
       <c r="Q59" s="4">
         <v>27</v>
       </c>
-      <c r="R59" s="46" t="s">
+      <c r="R59" s="4" t="s">
         <v>98</v>
       </c>
       <c r="S59" s="4" t="s">
@@ -19324,7 +19275,7 @@
       <c r="Q60" s="4">
         <v>990</v>
       </c>
-      <c r="R60" s="46" t="s">
+      <c r="R60" s="4" t="s">
         <v>108</v>
       </c>
       <c r="S60" s="4" t="s">
@@ -19389,7 +19340,7 @@
       <c r="Q61" s="4">
         <v>990</v>
       </c>
-      <c r="R61" s="46" t="s">
+      <c r="R61" s="4" t="s">
         <v>108</v>
       </c>
       <c r="S61" s="4" t="s">
@@ -19457,7 +19408,7 @@
       <c r="Q62" s="4">
         <v>990</v>
       </c>
-      <c r="R62" s="46" t="s">
+      <c r="R62" s="4" t="s">
         <v>108</v>
       </c>
       <c r="S62" s="4" t="s">
@@ -19525,7 +19476,7 @@
       <c r="Q63" s="4">
         <v>990</v>
       </c>
-      <c r="R63" s="46" t="s">
+      <c r="R63" s="4" t="s">
         <v>108</v>
       </c>
       <c r="S63" s="4" t="s">
@@ -19587,10 +19538,10 @@
       <c r="P64" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="Q64" s="35">
+      <c r="Q64" s="32">
         <v>146</v>
       </c>
-      <c r="R64" s="46">
+      <c r="R64" s="4">
         <v>9</v>
       </c>
       <c r="S64" s="4" t="s">
@@ -19604,136 +19555,136 @@
       </c>
     </row>
     <row r="65" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A65" s="35" t="s">
+      <c r="A65" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="B65" s="35">
+      <c r="B65" s="32">
         <v>1978</v>
       </c>
-      <c r="C65" s="35" t="s">
+      <c r="C65" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="D65" s="35" t="s">
+      <c r="D65" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="E65" s="35" t="s">
+      <c r="E65" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="F65" s="36">
+      <c r="F65" s="33">
         <v>1976</v>
       </c>
-      <c r="G65" s="37"/>
-      <c r="H65" s="35" t="s">
+      <c r="G65" s="34"/>
+      <c r="H65" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="I65" s="35" t="s">
+      <c r="I65" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="J65" s="36" t="s">
+      <c r="J65" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="K65" s="35">
+      <c r="K65" s="32">
         <v>1</v>
       </c>
-      <c r="L65" s="35" t="s">
+      <c r="L65" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="M65" s="35">
+      <c r="M65" s="32">
         <v>37</v>
       </c>
-      <c r="N65" s="35">
+      <c r="N65" s="32">
         <v>135</v>
       </c>
-      <c r="O65" s="35">
+      <c r="O65" s="32">
         <v>1103</v>
       </c>
-      <c r="P65" s="35" t="s">
+      <c r="P65" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="Q65" s="35">
+      <c r="Q65" s="32">
         <v>146</v>
       </c>
-      <c r="R65" s="46">
+      <c r="R65" s="4">
         <v>9</v>
       </c>
-      <c r="S65" s="35" t="s">
+      <c r="S65" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="T65" s="35" t="b">
+      <c r="T65" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U65" s="35" t="b">
+      <c r="U65" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="V65" s="40" t="s">
+      <c r="V65" s="37" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="66" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A66" s="38" t="s">
+      <c r="A66" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="B66" s="38">
+      <c r="B66" s="35">
         <v>1978</v>
       </c>
-      <c r="C66" s="38" t="s">
+      <c r="C66" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="D66" s="38" t="s">
+      <c r="D66" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="E66" s="38" t="s">
+      <c r="E66" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="F66" s="39">
+      <c r="F66" s="36">
         <v>1976</v>
       </c>
-      <c r="G66" s="38"/>
-      <c r="H66" s="38" t="s">
+      <c r="G66" s="35"/>
+      <c r="H66" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="I66" s="38" t="s">
+      <c r="I66" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="J66" s="39" t="s">
+      <c r="J66" s="36" t="s">
         <v>149</v>
       </c>
-      <c r="K66" s="38">
+      <c r="K66" s="35">
         <v>1</v>
       </c>
-      <c r="L66" s="38" t="s">
+      <c r="L66" s="35" t="s">
         <v>118</v>
       </c>
-      <c r="M66" s="38">
+      <c r="M66" s="35">
         <f>M64-M65</f>
         <v>25</v>
       </c>
-      <c r="N66" s="38">
+      <c r="N66" s="35">
         <f>O65-N65</f>
         <v>968</v>
       </c>
-      <c r="O66" s="38">
+      <c r="O66" s="35">
         <v>1103</v>
       </c>
-      <c r="P66" s="38" t="s">
+      <c r="P66" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="Q66" s="35">
+      <c r="Q66" s="32">
         <v>146</v>
       </c>
-      <c r="R66" s="46">
+      <c r="R66" s="4">
         <v>9</v>
       </c>
-      <c r="S66" s="38" t="s">
+      <c r="S66" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="T66" s="35" t="b">
+      <c r="T66" s="32" t="b">
         <v>0</v>
       </c>
-      <c r="U66" s="38" t="b">
+      <c r="U66" s="35" t="b">
         <v>1</v>
       </c>
-      <c r="V66" s="40" t="s">
+      <c r="V66" s="37" t="s">
         <v>202</v>
       </c>
     </row>
@@ -19786,7 +19737,7 @@
       <c r="Q67" s="4">
         <v>17</v>
       </c>
-      <c r="R67" s="46">
+      <c r="R67" s="4">
         <v>9</v>
       </c>
       <c r="S67" s="4" t="s">
@@ -19848,16 +19799,16 @@
       <c r="Q68" s="4">
         <v>17</v>
       </c>
-      <c r="R68" s="46">
+      <c r="R68" s="4">
         <v>9</v>
       </c>
-      <c r="S68" s="33" t="s">
+      <c r="S68" s="31" t="s">
         <v>125</v>
       </c>
-      <c r="T68" s="33" t="b">
+      <c r="T68" s="31" t="b">
         <v>0</v>
       </c>
-      <c r="U68" s="33" t="b">
+      <c r="U68" s="31" t="b">
         <v>0</v>
       </c>
       <c r="V68" s="29" t="s">
@@ -19914,16 +19865,16 @@
       <c r="Q69" s="4">
         <v>17</v>
       </c>
-      <c r="R69" s="46">
+      <c r="R69" s="4">
         <v>9</v>
       </c>
-      <c r="S69" s="33" t="s">
+      <c r="S69" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="T69" s="33" t="b">
+      <c r="T69" s="31" t="b">
         <v>1</v>
       </c>
-      <c r="U69" s="33" t="b">
+      <c r="U69" s="31" t="b">
         <v>1</v>
       </c>
     </row>
@@ -19976,7 +19927,7 @@
       <c r="Q70" s="4">
         <v>17</v>
       </c>
-      <c r="R70" s="46">
+      <c r="R70" s="4">
         <v>9</v>
       </c>
       <c r="S70" s="4" t="s">
@@ -20041,7 +19992,7 @@
       <c r="Q71" s="12">
         <v>123</v>
       </c>
-      <c r="R71" s="47" t="s">
+      <c r="R71" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S71" s="11" t="s">
@@ -20106,7 +20057,7 @@
       <c r="Q72" s="12">
         <v>123</v>
       </c>
-      <c r="R72" s="47" t="s">
+      <c r="R72" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S72" s="11" t="s">
@@ -20171,7 +20122,7 @@
       <c r="Q73" s="12">
         <v>123</v>
       </c>
-      <c r="R73" s="47" t="s">
+      <c r="R73" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S73" s="11" t="s">
@@ -20236,7 +20187,7 @@
       <c r="Q74" s="12">
         <v>123</v>
       </c>
-      <c r="R74" s="47" t="s">
+      <c r="R74" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S74" s="11" t="s">
@@ -20301,7 +20252,7 @@
       <c r="Q75" s="12">
         <v>123</v>
       </c>
-      <c r="R75" s="47" t="s">
+      <c r="R75" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S75" s="11" t="s">
@@ -20369,7 +20320,7 @@
       <c r="Q76" s="12">
         <v>123</v>
       </c>
-      <c r="R76" s="47" t="s">
+      <c r="R76" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S76" s="11" t="s">
@@ -20439,7 +20390,7 @@
       <c r="Q77" s="12">
         <v>123</v>
       </c>
-      <c r="R77" s="47" t="s">
+      <c r="R77" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S77" s="11" t="s">
@@ -20505,7 +20456,7 @@
       <c r="Q78" s="12">
         <v>123</v>
       </c>
-      <c r="R78" s="47" t="s">
+      <c r="R78" s="11" t="s">
         <v>133</v>
       </c>
       <c r="S78" s="11" t="s">
@@ -24347,7 +24298,7 @@
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
     <col min="2" max="2" width="11.1640625" customWidth="1"/>
     <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.6640625" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="39.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.5" bestFit="1" customWidth="1"/>
@@ -24412,7 +24363,7 @@
       <c r="G2" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="J2" s="32" t="s">
+      <c r="J2" s="4" t="s">
         <v>195</v>
       </c>
       <c r="K2" s="26"/>
@@ -24440,7 +24391,7 @@
       <c r="G3" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="J3" s="32" t="s">
+      <c r="J3" s="4" t="s">
         <v>195</v>
       </c>
       <c r="K3" s="26"/>
@@ -24459,13 +24410,13 @@
       <c r="D4" s="4">
         <v>1</v>
       </c>
-      <c r="E4" s="31" t="s">
+      <c r="E4" s="4" t="s">
         <v>28</v>
       </c>
       <c r="F4" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="J4" s="32" t="s">
+      <c r="J4" s="4" t="s">
         <v>195</v>
       </c>
       <c r="K4" s="26"/>
@@ -24499,7 +24450,7 @@
       <c r="I5" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="J5" s="34" t="s">
+      <c r="J5" s="17" t="s">
         <v>197</v>
       </c>
       <c r="K5" s="26"/>
@@ -24527,7 +24478,7 @@
       <c r="G6" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="J6" s="32" t="s">
+      <c r="J6" s="4" t="s">
         <v>198</v>
       </c>
       <c r="K6" s="26"/>
@@ -24558,7 +24509,7 @@
       <c r="H7" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="J7" s="32" t="s">
+      <c r="J7" s="4" t="s">
         <v>199</v>
       </c>
       <c r="K7" s="26"/>
@@ -24586,7 +24537,7 @@
       <c r="G8" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="J8" s="32" t="s">
+      <c r="J8" s="4" t="s">
         <v>199</v>
       </c>
     </row>
@@ -24629,7 +24580,7 @@
       <c r="E10" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="4" t="s">
         <v>159</v>
       </c>
     </row>
@@ -24649,7 +24600,7 @@
       <c r="E11" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="F11" s="32" t="s">
+      <c r="F11" s="4" t="s">
         <v>161</v>
       </c>
     </row>
@@ -24794,13 +24745,13 @@
       <c r="F19" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="G19" s="32" t="s">
+      <c r="G19" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="H19" s="32" t="s">
+      <c r="H19" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="I19" s="32" t="s">
+      <c r="I19" s="4" t="s">
         <v>130</v>
       </c>
     </row>
@@ -24859,7 +24810,7 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="14">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="31" t="s">
         <v>101</v>
       </c>
       <c r="B23" s="4" t="s">
@@ -24879,7 +24830,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="28">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="31" t="s">
         <v>101</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -24894,12 +24845,12 @@
       <c r="E24" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F24" s="32" t="s">
+      <c r="F24" s="4" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="14">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="31" t="s">
         <v>101</v>
       </c>
       <c r="B25" s="4" t="s">
@@ -24914,7 +24865,7 @@
       <c r="E25" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="F25" s="32" t="s">
+      <c r="F25" s="4" t="s">
         <v>157</v>
       </c>
     </row>
@@ -24968,13 +24919,13 @@
       <c r="E28" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="F28" s="32" t="s">
+      <c r="F28" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="G28" s="32" t="s">
+      <c r="G28" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="J28" s="32" t="s">
+      <c r="J28" s="4" t="s">
         <v>201</v>
       </c>
     </row>
@@ -24991,7 +24942,7 @@
       <c r="D29" s="4">
         <v>1</v>
       </c>
-      <c r="E29" s="33" t="s">
+      <c r="E29" s="31" t="s">
         <v>52</v>
       </c>
       <c r="F29" s="4" t="s">
@@ -29009,8 +28960,9 @@
       <c r="E1006" s="17"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="12" type="noConversion"/>
+  <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -29098,7 +29050,7 @@
         <v>186</v>
       </c>
       <c r="E3" s="27"/>
-      <c r="F3" s="43" t="s">
+      <c r="F3" s="38" t="s">
         <v>204</v>
       </c>
     </row>
@@ -35373,7 +35325,7 @@
       <c r="F2" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="I2" s="32" t="s">
+      <c r="I2" s="4" t="s">
         <v>195</v>
       </c>
     </row>
@@ -35396,7 +35348,7 @@
       <c r="F3" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="I3" s="32" t="s">
+      <c r="I3" s="4" t="s">
         <v>195</v>
       </c>
     </row>
@@ -35416,7 +35368,7 @@
       <c r="E4" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="I4" s="32" t="s">
+      <c r="I4" s="4" t="s">
         <v>195</v>
       </c>
     </row>
@@ -35445,7 +35397,7 @@
       <c r="H5" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="I5" s="34" t="s">
+      <c r="I5" s="17" t="s">
         <v>197</v>
       </c>
     </row>
@@ -35468,7 +35420,7 @@
       <c r="F6" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="4" t="s">
         <v>198</v>
       </c>
     </row>
@@ -35494,7 +35446,7 @@
       <c r="G7" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="I7" s="32" t="s">
+      <c r="I7" s="4" t="s">
         <v>199</v>
       </c>
     </row>
@@ -35517,7 +35469,7 @@
       <c r="F8" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="I8" s="32" t="s">
+      <c r="I8" s="4" t="s">
         <v>199</v>
       </c>
     </row>
@@ -35554,7 +35506,7 @@
       <c r="D10" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="E10" s="4" t="s">
         <v>159</v>
       </c>
     </row>
@@ -35571,7 +35523,7 @@
       <c r="D11" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="4" t="s">
         <v>161</v>
       </c>
     </row>
@@ -35690,7 +35642,7 @@
       <c r="D18" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="E18" s="32" t="s">
+      <c r="E18" s="4" t="s">
         <v>159</v>
       </c>
     </row>
@@ -35707,7 +35659,7 @@
       <c r="D19" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E19" s="32" t="s">
+      <c r="E19" s="4" t="s">
         <v>157</v>
       </c>
     </row>
@@ -35721,13 +35673,13 @@
       <c r="C20" s="5">
         <v>1976</v>
       </c>
-      <c r="D20" s="33" t="s">
+      <c r="D20" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="E20" s="32" t="s">
+      <c r="E20" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="32" t="s">
+      <c r="F20" s="4" t="s">
         <v>163</v>
       </c>
     </row>

</xml_diff>